<commit_message>
Fix navigation menu accessibility
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E670"/>
+  <dimension ref="A1:E671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13155,20 +13155,39 @@
     </row>
     <row r="670">
       <c r="A670" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C670" t="n">
+        <v>31</v>
+      </c>
+      <c r="D670" t="n">
+        <v>31</v>
+      </c>
+      <c r="E670" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B670" t="inlineStr">
+      <c r="B671" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C670" t="n">
-        <v>31</v>
-      </c>
-      <c r="D670" t="n">
-        <v>31</v>
-      </c>
-      <c r="E670" t="n">
+      <c r="C671" t="n">
+        <v>31</v>
+      </c>
+      <c r="D671" t="n">
+        <v>31</v>
+      </c>
+      <c r="E671" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13183,7 +13202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E670"/>
+  <dimension ref="A1:E671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25907,20 +25926,39 @@
     </row>
     <row r="670">
       <c r="A670" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C670" t="n">
+        <v>31</v>
+      </c>
+      <c r="D670" t="n">
+        <v>31</v>
+      </c>
+      <c r="E670" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B670" t="inlineStr">
+      <c r="B671" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C670" t="n">
-        <v>31</v>
-      </c>
-      <c r="D670" t="n">
-        <v>31</v>
-      </c>
-      <c r="E670" t="n">
+      <c r="C671" t="n">
+        <v>31</v>
+      </c>
+      <c r="D671" t="n">
+        <v>31</v>
+      </c>
+      <c r="E671" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Upgrade error message display
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E671"/>
+  <dimension ref="A1:E672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13174,20 +13174,39 @@
     </row>
     <row r="671">
       <c r="A671" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C671" t="n">
+        <v>31</v>
+      </c>
+      <c r="D671" t="n">
+        <v>31</v>
+      </c>
+      <c r="E671" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B671" t="inlineStr">
+      <c r="B672" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C671" t="n">
-        <v>31</v>
-      </c>
-      <c r="D671" t="n">
-        <v>31</v>
-      </c>
-      <c r="E671" t="n">
+      <c r="C672" t="n">
+        <v>31</v>
+      </c>
+      <c r="D672" t="n">
+        <v>31</v>
+      </c>
+      <c r="E672" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13202,7 +13221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E671"/>
+  <dimension ref="A1:E672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25945,20 +25964,39 @@
     </row>
     <row r="671">
       <c r="A671" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C671" t="n">
+        <v>31</v>
+      </c>
+      <c r="D671" t="n">
+        <v>31</v>
+      </c>
+      <c r="E671" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B671" t="inlineStr">
+      <c r="B672" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C671" t="n">
-        <v>31</v>
-      </c>
-      <c r="D671" t="n">
-        <v>31</v>
-      </c>
-      <c r="E671" t="n">
+      <c r="C672" t="n">
+        <v>31</v>
+      </c>
+      <c r="D672" t="n">
+        <v>31</v>
+      </c>
+      <c r="E672" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement data parsing logic
Add input validation for better security.
Remove deprecated functions and clean up codebase.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E672"/>
+  <dimension ref="A1:E673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13193,20 +13193,39 @@
     </row>
     <row r="672">
       <c r="A672" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>31</v>
+      </c>
+      <c r="D672" t="n">
+        <v>31</v>
+      </c>
+      <c r="E672" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B673" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C672" t="n">
-        <v>31</v>
-      </c>
-      <c r="D672" t="n">
-        <v>31</v>
-      </c>
-      <c r="E672" t="n">
+      <c r="C673" t="n">
+        <v>31</v>
+      </c>
+      <c r="D673" t="n">
+        <v>31</v>
+      </c>
+      <c r="E673" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13221,7 +13240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E672"/>
+  <dimension ref="A1:E673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25983,20 +26002,39 @@
     </row>
     <row r="672">
       <c r="A672" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C672" t="n">
+        <v>31</v>
+      </c>
+      <c r="D672" t="n">
+        <v>31</v>
+      </c>
+      <c r="E672" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B673" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C672" t="n">
-        <v>31</v>
-      </c>
-      <c r="D672" t="n">
-        <v>31</v>
-      </c>
-      <c r="E672" t="n">
+      <c r="C673" t="n">
+        <v>31</v>
+      </c>
+      <c r="D673" t="n">
+        <v>31</v>
+      </c>
+      <c r="E673" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust build script optimization
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E673"/>
+  <dimension ref="A1:E674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13212,20 +13212,39 @@
     </row>
     <row r="673">
       <c r="A673" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>31</v>
+      </c>
+      <c r="D673" t="n">
+        <v>31</v>
+      </c>
+      <c r="E673" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B673" t="inlineStr">
+      <c r="B674" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C673" t="n">
-        <v>31</v>
-      </c>
-      <c r="D673" t="n">
-        <v>31</v>
-      </c>
-      <c r="E673" t="n">
+      <c r="C674" t="n">
+        <v>31</v>
+      </c>
+      <c r="D674" t="n">
+        <v>31</v>
+      </c>
+      <c r="E674" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13240,7 +13259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E673"/>
+  <dimension ref="A1:E674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26021,20 +26040,39 @@
     </row>
     <row r="673">
       <c r="A673" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C673" t="n">
+        <v>31</v>
+      </c>
+      <c r="D673" t="n">
+        <v>31</v>
+      </c>
+      <c r="E673" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B673" t="inlineStr">
+      <c r="B674" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C673" t="n">
-        <v>31</v>
-      </c>
-      <c r="D673" t="n">
-        <v>31</v>
-      </c>
-      <c r="E673" t="n">
+      <c r="C674" t="n">
+        <v>31</v>
+      </c>
+      <c r="D674" t="n">
+        <v>31</v>
+      </c>
+      <c r="E674" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance login page ui elements
Apply code style fixes as per linter recommendations.
Improve performance by optimizing database queries.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E674"/>
+  <dimension ref="A1:E675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13231,20 +13231,39 @@
     </row>
     <row r="674">
       <c r="A674" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>31</v>
+      </c>
+      <c r="D674" t="n">
+        <v>31</v>
+      </c>
+      <c r="E674" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B674" t="inlineStr">
+      <c r="B675" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C674" t="n">
-        <v>31</v>
-      </c>
-      <c r="D674" t="n">
-        <v>31</v>
-      </c>
-      <c r="E674" t="n">
+      <c r="C675" t="n">
+        <v>31</v>
+      </c>
+      <c r="D675" t="n">
+        <v>31</v>
+      </c>
+      <c r="E675" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13259,7 +13278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E674"/>
+  <dimension ref="A1:E675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26059,20 +26078,39 @@
     </row>
     <row r="674">
       <c r="A674" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C674" t="n">
+        <v>31</v>
+      </c>
+      <c r="D674" t="n">
+        <v>31</v>
+      </c>
+      <c r="E674" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B674" t="inlineStr">
+      <c r="B675" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C674" t="n">
-        <v>31</v>
-      </c>
-      <c r="D674" t="n">
-        <v>31</v>
-      </c>
-      <c r="E674" t="n">
+      <c r="C675" t="n">
+        <v>31</v>
+      </c>
+      <c r="D675" t="n">
+        <v>31</v>
+      </c>
+      <c r="E675" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust navigation menu accessibility
Improve performance by optimizing database queries.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E675"/>
+  <dimension ref="A1:E676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13250,20 +13250,39 @@
     </row>
     <row r="675">
       <c r="A675" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>31</v>
+      </c>
+      <c r="D675" t="n">
+        <v>31</v>
+      </c>
+      <c r="E675" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B675" t="inlineStr">
+      <c r="B676" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C675" t="n">
-        <v>31</v>
-      </c>
-      <c r="D675" t="n">
-        <v>31</v>
-      </c>
-      <c r="E675" t="n">
+      <c r="C676" t="n">
+        <v>31</v>
+      </c>
+      <c r="D676" t="n">
+        <v>31</v>
+      </c>
+      <c r="E676" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13278,7 +13297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E675"/>
+  <dimension ref="A1:E676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26097,20 +26116,39 @@
     </row>
     <row r="675">
       <c r="A675" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C675" t="n">
+        <v>31</v>
+      </c>
+      <c r="D675" t="n">
+        <v>31</v>
+      </c>
+      <c r="E675" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B675" t="inlineStr">
+      <c r="B676" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C675" t="n">
-        <v>31</v>
-      </c>
-      <c r="D675" t="n">
-        <v>31</v>
-      </c>
-      <c r="E675" t="n">
+      <c r="C676" t="n">
+        <v>31</v>
+      </c>
+      <c r="D676" t="n">
+        <v>31</v>
+      </c>
+      <c r="E676" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify api response formatting
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E676"/>
+  <dimension ref="A1:E677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13269,20 +13269,39 @@
     </row>
     <row r="676">
       <c r="A676" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>31</v>
+      </c>
+      <c r="D676" t="n">
+        <v>31</v>
+      </c>
+      <c r="E676" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B676" t="inlineStr">
+      <c r="B677" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C676" t="n">
-        <v>31</v>
-      </c>
-      <c r="D676" t="n">
-        <v>31</v>
-      </c>
-      <c r="E676" t="n">
+      <c r="C677" t="n">
+        <v>31</v>
+      </c>
+      <c r="D677" t="n">
+        <v>31</v>
+      </c>
+      <c r="E677" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13297,7 +13316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E676"/>
+  <dimension ref="A1:E677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26135,20 +26154,39 @@
     </row>
     <row r="676">
       <c r="A676" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C676" t="n">
+        <v>31</v>
+      </c>
+      <c r="D676" t="n">
+        <v>31</v>
+      </c>
+      <c r="E676" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B676" t="inlineStr">
+      <c r="B677" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C676" t="n">
-        <v>31</v>
-      </c>
-      <c r="D676" t="n">
-        <v>31</v>
-      </c>
-      <c r="E676" t="n">
+      <c r="C677" t="n">
+        <v>31</v>
+      </c>
+      <c r="D677" t="n">
+        <v>31</v>
+      </c>
+      <c r="E677" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust login page ui elements
Remove deprecated functions and clean up codebase.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E677"/>
+  <dimension ref="A1:E678"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13288,20 +13288,39 @@
     </row>
     <row r="677">
       <c r="A677" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>31</v>
+      </c>
+      <c r="D677" t="n">
+        <v>31</v>
+      </c>
+      <c r="E677" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B677" t="inlineStr">
+      <c r="B678" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C677" t="n">
-        <v>31</v>
-      </c>
-      <c r="D677" t="n">
-        <v>31</v>
-      </c>
-      <c r="E677" t="n">
+      <c r="C678" t="n">
+        <v>31</v>
+      </c>
+      <c r="D678" t="n">
+        <v>31</v>
+      </c>
+      <c r="E678" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13316,7 +13335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E677"/>
+  <dimension ref="A1:E678"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26173,20 +26192,39 @@
     </row>
     <row r="677">
       <c r="A677" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C677" t="n">
+        <v>31</v>
+      </c>
+      <c r="D677" t="n">
+        <v>31</v>
+      </c>
+      <c r="E677" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B677" t="inlineStr">
+      <c r="B678" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C677" t="n">
-        <v>31</v>
-      </c>
-      <c r="D677" t="n">
-        <v>31</v>
-      </c>
-      <c r="E677" t="n">
+      <c r="C678" t="n">
+        <v>31</v>
+      </c>
+      <c r="D678" t="n">
+        <v>31</v>
+      </c>
+      <c r="E678" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct unit test coverage
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E678"/>
+  <dimension ref="A1:E679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13307,20 +13307,39 @@
     </row>
     <row r="678">
       <c r="A678" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>31</v>
+      </c>
+      <c r="D678" t="n">
+        <v>31</v>
+      </c>
+      <c r="E678" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B678" t="inlineStr">
+      <c r="B679" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C678" t="n">
-        <v>31</v>
-      </c>
-      <c r="D678" t="n">
-        <v>31</v>
-      </c>
-      <c r="E678" t="n">
+      <c r="C679" t="n">
+        <v>31</v>
+      </c>
+      <c r="D679" t="n">
+        <v>31</v>
+      </c>
+      <c r="E679" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13335,7 +13354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E678"/>
+  <dimension ref="A1:E679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26211,20 +26230,39 @@
     </row>
     <row r="678">
       <c r="A678" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C678" t="n">
+        <v>31</v>
+      </c>
+      <c r="D678" t="n">
+        <v>31</v>
+      </c>
+      <c r="E678" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B678" t="inlineStr">
+      <c r="B679" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C678" t="n">
-        <v>31</v>
-      </c>
-      <c r="D678" t="n">
-        <v>31</v>
-      </c>
-      <c r="E678" t="n">
+      <c r="C679" t="n">
+        <v>31</v>
+      </c>
+      <c r="D679" t="n">
+        <v>31</v>
+      </c>
+      <c r="E679" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Upgrade logging system configuration
Remove deprecated functions and clean up codebase.
Fix race condition in concurrent processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E679"/>
+  <dimension ref="A1:E680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13326,20 +13326,39 @@
     </row>
     <row r="679">
       <c r="A679" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>31</v>
+      </c>
+      <c r="D679" t="n">
+        <v>31</v>
+      </c>
+      <c r="E679" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B679" t="inlineStr">
+      <c r="B680" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C679" t="n">
-        <v>31</v>
-      </c>
-      <c r="D679" t="n">
-        <v>31</v>
-      </c>
-      <c r="E679" t="n">
+      <c r="C680" t="n">
+        <v>31</v>
+      </c>
+      <c r="D680" t="n">
+        <v>31</v>
+      </c>
+      <c r="E680" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13354,7 +13373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E679"/>
+  <dimension ref="A1:E680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26249,20 +26268,39 @@
     </row>
     <row r="679">
       <c r="A679" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C679" t="n">
+        <v>31</v>
+      </c>
+      <c r="D679" t="n">
+        <v>31</v>
+      </c>
+      <c r="E679" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B679" t="inlineStr">
+      <c r="B680" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C679" t="n">
-        <v>31</v>
-      </c>
-      <c r="D679" t="n">
-        <v>31</v>
-      </c>
-      <c r="E679" t="n">
+      <c r="C680" t="n">
+        <v>31</v>
+      </c>
+      <c r="D680" t="n">
+        <v>31</v>
+      </c>
+      <c r="E680" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify error message display
Update dependencies to their latest versions.
Fix various typos in comments and documentation.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E680"/>
+  <dimension ref="A1:E681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13345,20 +13345,39 @@
     </row>
     <row r="680">
       <c r="A680" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>31</v>
+      </c>
+      <c r="D680" t="n">
+        <v>31</v>
+      </c>
+      <c r="E680" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B680" t="inlineStr">
+      <c r="B681" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C680" t="n">
-        <v>31</v>
-      </c>
-      <c r="D680" t="n">
-        <v>31</v>
-      </c>
-      <c r="E680" t="n">
+      <c r="C681" t="n">
+        <v>31</v>
+      </c>
+      <c r="D681" t="n">
+        <v>31</v>
+      </c>
+      <c r="E681" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13373,7 +13392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E680"/>
+  <dimension ref="A1:E681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26287,20 +26306,39 @@
     </row>
     <row r="680">
       <c r="A680" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C680" t="n">
+        <v>31</v>
+      </c>
+      <c r="D680" t="n">
+        <v>31</v>
+      </c>
+      <c r="E680" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B680" t="inlineStr">
+      <c r="B681" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C680" t="n">
-        <v>31</v>
-      </c>
-      <c r="D680" t="n">
-        <v>31</v>
-      </c>
-      <c r="E680" t="n">
+      <c r="C681" t="n">
+        <v>31</v>
+      </c>
+      <c r="D681" t="n">
+        <v>31</v>
+      </c>
+      <c r="E681" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct config file handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E682"/>
+  <dimension ref="A1:E683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13383,20 +13383,39 @@
     </row>
     <row r="682">
       <c r="A682" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>31</v>
+      </c>
+      <c r="D682" t="n">
+        <v>31</v>
+      </c>
+      <c r="E682" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B682" t="inlineStr">
+      <c r="B683" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C682" t="n">
-        <v>31</v>
-      </c>
-      <c r="D682" t="n">
-        <v>31</v>
-      </c>
-      <c r="E682" t="n">
+      <c r="C683" t="n">
+        <v>31</v>
+      </c>
+      <c r="D683" t="n">
+        <v>31</v>
+      </c>
+      <c r="E683" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13411,7 +13430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E682"/>
+  <dimension ref="A1:E683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26363,20 +26382,39 @@
     </row>
     <row r="682">
       <c r="A682" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C682" t="n">
+        <v>31</v>
+      </c>
+      <c r="D682" t="n">
+        <v>31</v>
+      </c>
+      <c r="E682" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B682" t="inlineStr">
+      <c r="B683" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C682" t="n">
-        <v>31</v>
-      </c>
-      <c r="D682" t="n">
-        <v>31</v>
-      </c>
-      <c r="E682" t="n">
+      <c r="C683" t="n">
+        <v>31</v>
+      </c>
+      <c r="D683" t="n">
+        <v>31</v>
+      </c>
+      <c r="E683" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove csv module error handling
This resolves issue #20.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E683"/>
+  <dimension ref="A1:E684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13402,20 +13402,39 @@
     </row>
     <row r="683">
       <c r="A683" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>31</v>
+      </c>
+      <c r="D683" t="n">
+        <v>31</v>
+      </c>
+      <c r="E683" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B684" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C683" t="n">
-        <v>31</v>
-      </c>
-      <c r="D683" t="n">
-        <v>31</v>
-      </c>
-      <c r="E683" t="n">
+      <c r="C684" t="n">
+        <v>31</v>
+      </c>
+      <c r="D684" t="n">
+        <v>31</v>
+      </c>
+      <c r="E684" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13430,7 +13449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E683"/>
+  <dimension ref="A1:E684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26401,20 +26420,39 @@
     </row>
     <row r="683">
       <c r="A683" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C683" t="n">
+        <v>31</v>
+      </c>
+      <c r="D683" t="n">
+        <v>31</v>
+      </c>
+      <c r="E683" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B684" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C683" t="n">
-        <v>31</v>
-      </c>
-      <c r="D683" t="n">
-        <v>31</v>
-      </c>
-      <c r="E683" t="n">
+      <c r="C684" t="n">
+        <v>31</v>
+      </c>
+      <c r="D684" t="n">
+        <v>31</v>
+      </c>
+      <c r="E684" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve navigation menu accessibility
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E684"/>
+  <dimension ref="A1:E685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13421,20 +13421,39 @@
     </row>
     <row r="684">
       <c r="A684" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>31</v>
+      </c>
+      <c r="D684" t="n">
+        <v>31</v>
+      </c>
+      <c r="E684" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B684" t="inlineStr">
+      <c r="B685" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C684" t="n">
-        <v>31</v>
-      </c>
-      <c r="D684" t="n">
-        <v>31</v>
-      </c>
-      <c r="E684" t="n">
+      <c r="C685" t="n">
+        <v>31</v>
+      </c>
+      <c r="D685" t="n">
+        <v>31</v>
+      </c>
+      <c r="E685" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13449,7 +13468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E684"/>
+  <dimension ref="A1:E685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26439,20 +26458,39 @@
     </row>
     <row r="684">
       <c r="A684" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C684" t="n">
+        <v>31</v>
+      </c>
+      <c r="D684" t="n">
+        <v>31</v>
+      </c>
+      <c r="E684" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B684" t="inlineStr">
+      <c r="B685" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C684" t="n">
-        <v>31</v>
-      </c>
-      <c r="D684" t="n">
-        <v>31</v>
-      </c>
-      <c r="E684" t="n">
+      <c r="C685" t="n">
+        <v>31</v>
+      </c>
+      <c r="D685" t="n">
+        <v>31</v>
+      </c>
+      <c r="E685" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement user authentication module
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E685"/>
+  <dimension ref="A1:E686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13440,20 +13440,39 @@
     </row>
     <row r="685">
       <c r="A685" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>31</v>
+      </c>
+      <c r="D685" t="n">
+        <v>31</v>
+      </c>
+      <c r="E685" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B685" t="inlineStr">
+      <c r="B686" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C685" t="n">
-        <v>31</v>
-      </c>
-      <c r="D685" t="n">
-        <v>31</v>
-      </c>
-      <c r="E685" t="n">
+      <c r="C686" t="n">
+        <v>31</v>
+      </c>
+      <c r="D686" t="n">
+        <v>31</v>
+      </c>
+      <c r="E686" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13468,7 +13487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E685"/>
+  <dimension ref="A1:E686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26477,20 +26496,39 @@
     </row>
     <row r="685">
       <c r="A685" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C685" t="n">
+        <v>31</v>
+      </c>
+      <c r="D685" t="n">
+        <v>31</v>
+      </c>
+      <c r="E685" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B685" t="inlineStr">
+      <c r="B686" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C685" t="n">
-        <v>31</v>
-      </c>
-      <c r="D685" t="n">
-        <v>31</v>
-      </c>
-      <c r="E685" t="n">
+      <c r="C686" t="n">
+        <v>31</v>
+      </c>
+      <c r="D686" t="n">
+        <v>31</v>
+      </c>
+      <c r="E686" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify responsive design implementation
Fix race condition in concurrent processing.
Remove deprecated functions and clean up codebase.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E687"/>
+  <dimension ref="A1:E688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13478,20 +13478,39 @@
     </row>
     <row r="687">
       <c r="A687" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>31</v>
+      </c>
+      <c r="D687" t="n">
+        <v>31</v>
+      </c>
+      <c r="E687" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B687" t="inlineStr">
+      <c r="B688" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C687" t="n">
-        <v>31</v>
-      </c>
-      <c r="D687" t="n">
-        <v>31</v>
-      </c>
-      <c r="E687" t="n">
+      <c r="C688" t="n">
+        <v>31</v>
+      </c>
+      <c r="D688" t="n">
+        <v>31</v>
+      </c>
+      <c r="E688" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13506,7 +13525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E687"/>
+  <dimension ref="A1:E688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26553,20 +26572,39 @@
     </row>
     <row r="687">
       <c r="A687" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C687" t="n">
+        <v>31</v>
+      </c>
+      <c r="D687" t="n">
+        <v>31</v>
+      </c>
+      <c r="E687" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B687" t="inlineStr">
+      <c r="B688" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C687" t="n">
-        <v>31</v>
-      </c>
-      <c r="D687" t="n">
-        <v>31</v>
-      </c>
-      <c r="E687" t="n">
+      <c r="C688" t="n">
+        <v>31</v>
+      </c>
+      <c r="D688" t="n">
+        <v>31</v>
+      </c>
+      <c r="E688" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance error message display
Enhance test coverage to prevent regressions.
Address edge cases reported in user feedback.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E688"/>
+  <dimension ref="A1:E689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13497,20 +13497,39 @@
     </row>
     <row r="688">
       <c r="A688" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C688" t="n">
+        <v>31</v>
+      </c>
+      <c r="D688" t="n">
+        <v>31</v>
+      </c>
+      <c r="E688" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B688" t="inlineStr">
+      <c r="B689" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C688" t="n">
-        <v>31</v>
-      </c>
-      <c r="D688" t="n">
-        <v>31</v>
-      </c>
-      <c r="E688" t="n">
+      <c r="C689" t="n">
+        <v>31</v>
+      </c>
+      <c r="D689" t="n">
+        <v>31</v>
+      </c>
+      <c r="E689" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13525,7 +13544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E688"/>
+  <dimension ref="A1:E689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26591,20 +26610,39 @@
     </row>
     <row r="688">
       <c r="A688" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C688" t="n">
+        <v>31</v>
+      </c>
+      <c r="D688" t="n">
+        <v>31</v>
+      </c>
+      <c r="E688" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B688" t="inlineStr">
+      <c r="B689" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C688" t="n">
-        <v>31</v>
-      </c>
-      <c r="D688" t="n">
-        <v>31</v>
-      </c>
-      <c r="E688" t="n">
+      <c r="C689" t="n">
+        <v>31</v>
+      </c>
+      <c r="D689" t="n">
+        <v>31</v>
+      </c>
+      <c r="E689" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix login page ui elements
Update dependencies to their latest versions.
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E689"/>
+  <dimension ref="A1:E690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13516,20 +13516,39 @@
     </row>
     <row r="689">
       <c r="A689" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C689" t="n">
+        <v>31</v>
+      </c>
+      <c r="D689" t="n">
+        <v>31</v>
+      </c>
+      <c r="E689" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B689" t="inlineStr">
+      <c r="B690" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C689" t="n">
-        <v>31</v>
-      </c>
-      <c r="D689" t="n">
-        <v>31</v>
-      </c>
-      <c r="E689" t="n">
+      <c r="C690" t="n">
+        <v>31</v>
+      </c>
+      <c r="D690" t="n">
+        <v>31</v>
+      </c>
+      <c r="E690" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13544,7 +13563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E689"/>
+  <dimension ref="A1:E690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26629,20 +26648,39 @@
     </row>
     <row r="689">
       <c r="A689" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C689" t="n">
+        <v>31</v>
+      </c>
+      <c r="D689" t="n">
+        <v>31</v>
+      </c>
+      <c r="E689" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B689" t="inlineStr">
+      <c r="B690" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C689" t="n">
-        <v>31</v>
-      </c>
-      <c r="D689" t="n">
-        <v>31</v>
-      </c>
-      <c r="E689" t="n">
+      <c r="C690" t="n">
+        <v>31</v>
+      </c>
+      <c r="D690" t="n">
+        <v>31</v>
+      </c>
+      <c r="E690" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize api endpoint validation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E690"/>
+  <dimension ref="A1:E691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13535,20 +13535,39 @@
     </row>
     <row r="690">
       <c r="A690" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C690" t="n">
+        <v>31</v>
+      </c>
+      <c r="D690" t="n">
+        <v>31</v>
+      </c>
+      <c r="E690" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B690" t="inlineStr">
+      <c r="B691" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C690" t="n">
-        <v>31</v>
-      </c>
-      <c r="D690" t="n">
-        <v>31</v>
-      </c>
-      <c r="E690" t="n">
+      <c r="C691" t="n">
+        <v>31</v>
+      </c>
+      <c r="D691" t="n">
+        <v>31</v>
+      </c>
+      <c r="E691" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13563,7 +13582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E690"/>
+  <dimension ref="A1:E691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26667,20 +26686,39 @@
     </row>
     <row r="690">
       <c r="A690" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C690" t="n">
+        <v>31</v>
+      </c>
+      <c r="D690" t="n">
+        <v>31</v>
+      </c>
+      <c r="E690" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B690" t="inlineStr">
+      <c r="B691" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C690" t="n">
-        <v>31</v>
-      </c>
-      <c r="D690" t="n">
-        <v>31</v>
-      </c>
-      <c r="E690" t="n">
+      <c r="C691" t="n">
+        <v>31</v>
+      </c>
+      <c r="D691" t="n">
+        <v>31</v>
+      </c>
+      <c r="E691" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance config file handling
Fix race condition in concurrent processing.
Refactor legacy code to follow modern practices.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E691"/>
+  <dimension ref="A1:E692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13554,20 +13554,39 @@
     </row>
     <row r="691">
       <c r="A691" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>31</v>
+      </c>
+      <c r="D691" t="n">
+        <v>31</v>
+      </c>
+      <c r="E691" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B691" t="inlineStr">
+      <c r="B692" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C691" t="n">
-        <v>31</v>
-      </c>
-      <c r="D691" t="n">
-        <v>31</v>
-      </c>
-      <c r="E691" t="n">
+      <c r="C692" t="n">
+        <v>31</v>
+      </c>
+      <c r="D692" t="n">
+        <v>31</v>
+      </c>
+      <c r="E692" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13582,7 +13601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E691"/>
+  <dimension ref="A1:E692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26705,20 +26724,39 @@
     </row>
     <row r="691">
       <c r="A691" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>31</v>
+      </c>
+      <c r="D691" t="n">
+        <v>31</v>
+      </c>
+      <c r="E691" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B691" t="inlineStr">
+      <c r="B692" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C691" t="n">
-        <v>31</v>
-      </c>
-      <c r="D691" t="n">
-        <v>31</v>
-      </c>
-      <c r="E691" t="n">
+      <c r="C692" t="n">
+        <v>31</v>
+      </c>
+      <c r="D692" t="n">
+        <v>31</v>
+      </c>
+      <c r="E692" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E692"/>
+  <dimension ref="A1:E693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13573,20 +13573,39 @@
     </row>
     <row r="692">
       <c r="A692" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>31</v>
+      </c>
+      <c r="D692" t="n">
+        <v>31</v>
+      </c>
+      <c r="E692" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B692" t="inlineStr">
+      <c r="B693" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C692" t="n">
-        <v>31</v>
-      </c>
-      <c r="D692" t="n">
-        <v>31</v>
-      </c>
-      <c r="E692" t="n">
+      <c r="C693" t="n">
+        <v>31</v>
+      </c>
+      <c r="D693" t="n">
+        <v>31</v>
+      </c>
+      <c r="E693" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13601,7 +13620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E692"/>
+  <dimension ref="A1:E693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26743,20 +26762,39 @@
     </row>
     <row r="692">
       <c r="A692" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>31</v>
+      </c>
+      <c r="D692" t="n">
+        <v>31</v>
+      </c>
+      <c r="E692" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B692" t="inlineStr">
+      <c r="B693" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C692" t="n">
-        <v>31</v>
-      </c>
-      <c r="D692" t="n">
-        <v>31</v>
-      </c>
-      <c r="E692" t="n">
+      <c r="C693" t="n">
+        <v>31</v>
+      </c>
+      <c r="D693" t="n">
+        <v>31</v>
+      </c>
+      <c r="E693" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove api endpoint validation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E696"/>
+  <dimension ref="A1:E697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13649,20 +13649,39 @@
     </row>
     <row r="696">
       <c r="A696" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>31</v>
+      </c>
+      <c r="D696" t="n">
+        <v>31</v>
+      </c>
+      <c r="E696" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B696" t="inlineStr">
+      <c r="B697" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C696" t="n">
-        <v>31</v>
-      </c>
-      <c r="D696" t="n">
-        <v>31</v>
-      </c>
-      <c r="E696" t="n">
+      <c r="C697" t="n">
+        <v>31</v>
+      </c>
+      <c r="D697" t="n">
+        <v>31</v>
+      </c>
+      <c r="E697" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13677,7 +13696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E696"/>
+  <dimension ref="A1:E697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26895,20 +26914,39 @@
     </row>
     <row r="696">
       <c r="A696" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>31</v>
+      </c>
+      <c r="D696" t="n">
+        <v>31</v>
+      </c>
+      <c r="E696" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B696" t="inlineStr">
+      <c r="B697" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C696" t="n">
-        <v>31</v>
-      </c>
-      <c r="D696" t="n">
-        <v>31</v>
-      </c>
-      <c r="E696" t="n">
+      <c r="C697" t="n">
+        <v>31</v>
+      </c>
+      <c r="D697" t="n">
+        <v>31</v>
+      </c>
+      <c r="E697" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct database schema migration
Update dependencies to their latest versions.
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E697"/>
+  <dimension ref="A1:E698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13668,20 +13668,39 @@
     </row>
     <row r="697">
       <c r="A697" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>31</v>
+      </c>
+      <c r="D697" t="n">
+        <v>31</v>
+      </c>
+      <c r="E697" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B697" t="inlineStr">
+      <c r="B698" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C697" t="n">
-        <v>31</v>
-      </c>
-      <c r="D697" t="n">
-        <v>31</v>
-      </c>
-      <c r="E697" t="n">
+      <c r="C698" t="n">
+        <v>31</v>
+      </c>
+      <c r="D698" t="n">
+        <v>31</v>
+      </c>
+      <c r="E698" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13696,7 +13715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E697"/>
+  <dimension ref="A1:E698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26933,20 +26952,39 @@
     </row>
     <row r="697">
       <c r="A697" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>31</v>
+      </c>
+      <c r="D697" t="n">
+        <v>31</v>
+      </c>
+      <c r="E697" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B697" t="inlineStr">
+      <c r="B698" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C697" t="n">
-        <v>31</v>
-      </c>
-      <c r="D697" t="n">
-        <v>31</v>
-      </c>
-      <c r="E697" t="n">
+      <c r="C698" t="n">
+        <v>31</v>
+      </c>
+      <c r="D698" t="n">
+        <v>31</v>
+      </c>
+      <c r="E698" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E698"/>
+  <dimension ref="A1:E699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13687,20 +13687,39 @@
     </row>
     <row r="698">
       <c r="A698" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>31</v>
+      </c>
+      <c r="D698" t="n">
+        <v>31</v>
+      </c>
+      <c r="E698" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B698" t="inlineStr">
+      <c r="B699" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C698" t="n">
-        <v>31</v>
-      </c>
-      <c r="D698" t="n">
-        <v>31</v>
-      </c>
-      <c r="E698" t="n">
+      <c r="C699" t="n">
+        <v>31</v>
+      </c>
+      <c r="D699" t="n">
+        <v>31</v>
+      </c>
+      <c r="E699" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13715,7 +13734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E698"/>
+  <dimension ref="A1:E699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26971,20 +26990,39 @@
     </row>
     <row r="698">
       <c r="A698" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>31</v>
+      </c>
+      <c r="D698" t="n">
+        <v>31</v>
+      </c>
+      <c r="E698" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B698" t="inlineStr">
+      <c r="B699" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C698" t="n">
-        <v>31</v>
-      </c>
-      <c r="D698" t="n">
-        <v>31</v>
-      </c>
-      <c r="E698" t="n">
+      <c r="C699" t="n">
+        <v>31</v>
+      </c>
+      <c r="D699" t="n">
+        <v>31</v>
+      </c>
+      <c r="E699" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E699"/>
+  <dimension ref="A1:E700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13706,20 +13706,39 @@
     </row>
     <row r="699">
       <c r="A699" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>31</v>
+      </c>
+      <c r="D699" t="n">
+        <v>31</v>
+      </c>
+      <c r="E699" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B699" t="inlineStr">
+      <c r="B700" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C699" t="n">
-        <v>31</v>
-      </c>
-      <c r="D699" t="n">
-        <v>31</v>
-      </c>
-      <c r="E699" t="n">
+      <c r="C700" t="n">
+        <v>31</v>
+      </c>
+      <c r="D700" t="n">
+        <v>31</v>
+      </c>
+      <c r="E700" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13734,7 +13753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E699"/>
+  <dimension ref="A1:E700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27009,20 +27028,39 @@
     </row>
     <row r="699">
       <c r="A699" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>31</v>
+      </c>
+      <c r="D699" t="n">
+        <v>31</v>
+      </c>
+      <c r="E699" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B699" t="inlineStr">
+      <c r="B700" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C699" t="n">
-        <v>31</v>
-      </c>
-      <c r="D699" t="n">
-        <v>31</v>
-      </c>
-      <c r="E699" t="n">
+      <c r="C700" t="n">
+        <v>31</v>
+      </c>
+      <c r="D700" t="n">
+        <v>31</v>
+      </c>
+      <c r="E700" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct build script optimization
Add input validation for better security.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E702"/>
+  <dimension ref="A1:E703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13763,20 +13763,39 @@
     </row>
     <row r="702">
       <c r="A702" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>31</v>
+      </c>
+      <c r="D702" t="n">
+        <v>31</v>
+      </c>
+      <c r="E702" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B702" t="inlineStr">
+      <c r="B703" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C702" t="n">
-        <v>31</v>
-      </c>
-      <c r="D702" t="n">
-        <v>31</v>
-      </c>
-      <c r="E702" t="n">
+      <c r="C703" t="n">
+        <v>31</v>
+      </c>
+      <c r="D703" t="n">
+        <v>31</v>
+      </c>
+      <c r="E703" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13791,7 +13810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E702"/>
+  <dimension ref="A1:E703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27123,20 +27142,39 @@
     </row>
     <row r="702">
       <c r="A702" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>31</v>
+      </c>
+      <c r="D702" t="n">
+        <v>31</v>
+      </c>
+      <c r="E702" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B702" t="inlineStr">
+      <c r="B703" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C702" t="n">
-        <v>31</v>
-      </c>
-      <c r="D702" t="n">
-        <v>31</v>
-      </c>
-      <c r="E702" t="n">
+      <c r="C703" t="n">
+        <v>31</v>
+      </c>
+      <c r="D703" t="n">
+        <v>31</v>
+      </c>
+      <c r="E703" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove user authentication module
Enhance test coverage to prevent regressions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E703"/>
+  <dimension ref="A1:E704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13782,20 +13782,39 @@
     </row>
     <row r="703">
       <c r="A703" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>31</v>
+      </c>
+      <c r="D703" t="n">
+        <v>31</v>
+      </c>
+      <c r="E703" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B703" t="inlineStr">
+      <c r="B704" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C703" t="n">
-        <v>31</v>
-      </c>
-      <c r="D703" t="n">
-        <v>31</v>
-      </c>
-      <c r="E703" t="n">
+      <c r="C704" t="n">
+        <v>31</v>
+      </c>
+      <c r="D704" t="n">
+        <v>31</v>
+      </c>
+      <c r="E704" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13810,7 +13829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E703"/>
+  <dimension ref="A1:E704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27161,20 +27180,39 @@
     </row>
     <row r="703">
       <c r="A703" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>31</v>
+      </c>
+      <c r="D703" t="n">
+        <v>31</v>
+      </c>
+      <c r="E703" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B703" t="inlineStr">
+      <c r="B704" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C703" t="n">
-        <v>31</v>
-      </c>
-      <c r="D703" t="n">
-        <v>31</v>
-      </c>
-      <c r="E703" t="n">
+      <c r="C704" t="n">
+        <v>31</v>
+      </c>
+      <c r="D704" t="n">
+        <v>31</v>
+      </c>
+      <c r="E704" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise file upload functionality
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E705"/>
+  <dimension ref="A1:E706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13820,20 +13820,39 @@
     </row>
     <row r="705">
       <c r="A705" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>31</v>
+      </c>
+      <c r="D705" t="n">
+        <v>31</v>
+      </c>
+      <c r="E705" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B705" t="inlineStr">
+      <c r="B706" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C705" t="n">
-        <v>31</v>
-      </c>
-      <c r="D705" t="n">
-        <v>31</v>
-      </c>
-      <c r="E705" t="n">
+      <c r="C706" t="n">
+        <v>31</v>
+      </c>
+      <c r="D706" t="n">
+        <v>31</v>
+      </c>
+      <c r="E706" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13848,7 +13867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E705"/>
+  <dimension ref="A1:E706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27237,20 +27256,39 @@
     </row>
     <row r="705">
       <c r="A705" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>31</v>
+      </c>
+      <c r="D705" t="n">
+        <v>31</v>
+      </c>
+      <c r="E705" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B705" t="inlineStr">
+      <c r="B706" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C705" t="n">
-        <v>31</v>
-      </c>
-      <c r="D705" t="n">
-        <v>31</v>
-      </c>
-      <c r="E705" t="n">
+      <c r="C706" t="n">
+        <v>31</v>
+      </c>
+      <c r="D706" t="n">
+        <v>31</v>
+      </c>
+      <c r="E706" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify build script optimization
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E708"/>
+  <dimension ref="A1:E709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13877,20 +13877,39 @@
     </row>
     <row r="708">
       <c r="A708" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>31</v>
+      </c>
+      <c r="D708" t="n">
+        <v>31</v>
+      </c>
+      <c r="E708" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B708" t="inlineStr">
+      <c r="B709" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C708" t="n">
-        <v>31</v>
-      </c>
-      <c r="D708" t="n">
-        <v>31</v>
-      </c>
-      <c r="E708" t="n">
+      <c r="C709" t="n">
+        <v>31</v>
+      </c>
+      <c r="D709" t="n">
+        <v>31</v>
+      </c>
+      <c r="E709" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13905,7 +13924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E708"/>
+  <dimension ref="A1:E709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27351,20 +27370,39 @@
     </row>
     <row r="708">
       <c r="A708" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>31</v>
+      </c>
+      <c r="D708" t="n">
+        <v>31</v>
+      </c>
+      <c r="E708" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B708" t="inlineStr">
+      <c r="B709" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C708" t="n">
-        <v>31</v>
-      </c>
-      <c r="D708" t="n">
-        <v>31</v>
-      </c>
-      <c r="E708" t="n">
+      <c r="C709" t="n">
+        <v>31</v>
+      </c>
+      <c r="D709" t="n">
+        <v>31</v>
+      </c>
+      <c r="E709" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert database schema migration
Address edge cases reported in user feedback.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E709"/>
+  <dimension ref="A1:E710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13896,20 +13896,39 @@
     </row>
     <row r="709">
       <c r="A709" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>31</v>
+      </c>
+      <c r="D709" t="n">
+        <v>31</v>
+      </c>
+      <c r="E709" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B709" t="inlineStr">
+      <c r="B710" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C709" t="n">
-        <v>31</v>
-      </c>
-      <c r="D709" t="n">
-        <v>31</v>
-      </c>
-      <c r="E709" t="n">
+      <c r="C710" t="n">
+        <v>31</v>
+      </c>
+      <c r="D710" t="n">
+        <v>31</v>
+      </c>
+      <c r="E710" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13924,7 +13943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E709"/>
+  <dimension ref="A1:E710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27389,20 +27408,39 @@
     </row>
     <row r="709">
       <c r="A709" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>31</v>
+      </c>
+      <c r="D709" t="n">
+        <v>31</v>
+      </c>
+      <c r="E709" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B709" t="inlineStr">
+      <c r="B710" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C709" t="n">
-        <v>31</v>
-      </c>
-      <c r="D709" t="n">
-        <v>31</v>
-      </c>
-      <c r="E709" t="n">
+      <c r="C710" t="n">
+        <v>31</v>
+      </c>
+      <c r="D710" t="n">
+        <v>31</v>
+      </c>
+      <c r="E710" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E710"/>
+  <dimension ref="A1:E711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13915,20 +13915,39 @@
     </row>
     <row r="710">
       <c r="A710" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>31</v>
+      </c>
+      <c r="D710" t="n">
+        <v>31</v>
+      </c>
+      <c r="E710" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B710" t="inlineStr">
+      <c r="B711" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C710" t="n">
-        <v>31</v>
-      </c>
-      <c r="D710" t="n">
-        <v>31</v>
-      </c>
-      <c r="E710" t="n">
+      <c r="C711" t="n">
+        <v>31</v>
+      </c>
+      <c r="D711" t="n">
+        <v>31</v>
+      </c>
+      <c r="E711" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13943,7 +13962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E710"/>
+  <dimension ref="A1:E711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27427,20 +27446,39 @@
     </row>
     <row r="710">
       <c r="A710" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>31</v>
+      </c>
+      <c r="D710" t="n">
+        <v>31</v>
+      </c>
+      <c r="E710" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B710" t="inlineStr">
+      <c r="B711" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C710" t="n">
-        <v>31</v>
-      </c>
-      <c r="D710" t="n">
-        <v>31</v>
-      </c>
-      <c r="E710" t="n">
+      <c r="C711" t="n">
+        <v>31</v>
+      </c>
+      <c r="D711" t="n">
+        <v>31</v>
+      </c>
+      <c r="E711" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix database schema migration
Enhance test coverage to prevent regressions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E711"/>
+  <dimension ref="A1:E712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13934,20 +13934,39 @@
     </row>
     <row r="711">
       <c r="A711" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>31</v>
+      </c>
+      <c r="D711" t="n">
+        <v>31</v>
+      </c>
+      <c r="E711" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B711" t="inlineStr">
+      <c r="B712" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C711" t="n">
-        <v>31</v>
-      </c>
-      <c r="D711" t="n">
-        <v>31</v>
-      </c>
-      <c r="E711" t="n">
+      <c r="C712" t="n">
+        <v>31</v>
+      </c>
+      <c r="D712" t="n">
+        <v>31</v>
+      </c>
+      <c r="E712" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13962,7 +13981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E711"/>
+  <dimension ref="A1:E712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27465,20 +27484,39 @@
     </row>
     <row r="711">
       <c r="A711" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>31</v>
+      </c>
+      <c r="D711" t="n">
+        <v>31</v>
+      </c>
+      <c r="E711" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B711" t="inlineStr">
+      <c r="B712" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C711" t="n">
-        <v>31</v>
-      </c>
-      <c r="D711" t="n">
-        <v>31</v>
-      </c>
-      <c r="E711" t="n">
+      <c r="C712" t="n">
+        <v>31</v>
+      </c>
+      <c r="D712" t="n">
+        <v>31</v>
+      </c>
+      <c r="E712" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust responsive design implementation
This resolves issue #30.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E712"/>
+  <dimension ref="A1:E713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13953,20 +13953,39 @@
     </row>
     <row r="712">
       <c r="A712" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>31</v>
+      </c>
+      <c r="D712" t="n">
+        <v>31</v>
+      </c>
+      <c r="E712" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B712" t="inlineStr">
+      <c r="B713" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C712" t="n">
-        <v>31</v>
-      </c>
-      <c r="D712" t="n">
-        <v>31</v>
-      </c>
-      <c r="E712" t="n">
+      <c r="C713" t="n">
+        <v>31</v>
+      </c>
+      <c r="D713" t="n">
+        <v>31</v>
+      </c>
+      <c r="E713" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13981,7 +14000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E712"/>
+  <dimension ref="A1:E713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27503,20 +27522,39 @@
     </row>
     <row r="712">
       <c r="A712" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>31</v>
+      </c>
+      <c r="D712" t="n">
+        <v>31</v>
+      </c>
+      <c r="E712" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B712" t="inlineStr">
+      <c r="B713" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C712" t="n">
-        <v>31</v>
-      </c>
-      <c r="D712" t="n">
-        <v>31</v>
-      </c>
-      <c r="E712" t="n">
+      <c r="C713" t="n">
+        <v>31</v>
+      </c>
+      <c r="D713" t="n">
+        <v>31</v>
+      </c>
+      <c r="E713" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix logging system configuration
Fix race condition in concurrent processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E713"/>
+  <dimension ref="A1:E714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13972,20 +13972,39 @@
     </row>
     <row r="713">
       <c r="A713" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>31</v>
+      </c>
+      <c r="D713" t="n">
+        <v>31</v>
+      </c>
+      <c r="E713" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B713" t="inlineStr">
+      <c r="B714" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C713" t="n">
-        <v>31</v>
-      </c>
-      <c r="D713" t="n">
-        <v>31</v>
-      </c>
-      <c r="E713" t="n">
+      <c r="C714" t="n">
+        <v>31</v>
+      </c>
+      <c r="D714" t="n">
+        <v>31</v>
+      </c>
+      <c r="E714" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14000,7 +14019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E713"/>
+  <dimension ref="A1:E714"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27541,20 +27560,39 @@
     </row>
     <row r="713">
       <c r="A713" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>31</v>
+      </c>
+      <c r="D713" t="n">
+        <v>31</v>
+      </c>
+      <c r="E713" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B713" t="inlineStr">
+      <c r="B714" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C713" t="n">
-        <v>31</v>
-      </c>
-      <c r="D713" t="n">
-        <v>31</v>
-      </c>
-      <c r="E713" t="n">
+      <c r="C714" t="n">
+        <v>31</v>
+      </c>
+      <c r="D714" t="n">
+        <v>31</v>
+      </c>
+      <c r="E714" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E714"/>
+  <dimension ref="A1:E715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13991,20 +13991,39 @@
     </row>
     <row r="714">
       <c r="A714" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>31</v>
+      </c>
+      <c r="D714" t="n">
+        <v>31</v>
+      </c>
+      <c r="E714" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B714" t="inlineStr">
+      <c r="B715" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C714" t="n">
-        <v>31</v>
-      </c>
-      <c r="D714" t="n">
-        <v>31</v>
-      </c>
-      <c r="E714" t="n">
+      <c r="C715" t="n">
+        <v>31</v>
+      </c>
+      <c r="D715" t="n">
+        <v>31</v>
+      </c>
+      <c r="E715" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14019,7 +14038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E714"/>
+  <dimension ref="A1:E715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27579,20 +27598,39 @@
     </row>
     <row r="714">
       <c r="A714" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>31</v>
+      </c>
+      <c r="D714" t="n">
+        <v>31</v>
+      </c>
+      <c r="E714" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B714" t="inlineStr">
+      <c r="B715" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C714" t="n">
-        <v>31</v>
-      </c>
-      <c r="D714" t="n">
-        <v>31</v>
-      </c>
-      <c r="E714" t="n">
+      <c r="C715" t="n">
+        <v>31</v>
+      </c>
+      <c r="D715" t="n">
+        <v>31</v>
+      </c>
+      <c r="E715" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E715"/>
+  <dimension ref="A1:E716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14010,20 +14010,39 @@
     </row>
     <row r="715">
       <c r="A715" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>31</v>
+      </c>
+      <c r="D715" t="n">
+        <v>31</v>
+      </c>
+      <c r="E715" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B715" t="inlineStr">
+      <c r="B716" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C715" t="n">
-        <v>31</v>
-      </c>
-      <c r="D715" t="n">
-        <v>31</v>
-      </c>
-      <c r="E715" t="n">
+      <c r="C716" t="n">
+        <v>31</v>
+      </c>
+      <c r="D716" t="n">
+        <v>31</v>
+      </c>
+      <c r="E716" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14038,7 +14057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E715"/>
+  <dimension ref="A1:E716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27617,20 +27636,39 @@
     </row>
     <row r="715">
       <c r="A715" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>31</v>
+      </c>
+      <c r="D715" t="n">
+        <v>31</v>
+      </c>
+      <c r="E715" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B715" t="inlineStr">
+      <c r="B716" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C715" t="n">
-        <v>31</v>
-      </c>
-      <c r="D715" t="n">
-        <v>31</v>
-      </c>
-      <c r="E715" t="n">
+      <c r="C716" t="n">
+        <v>31</v>
+      </c>
+      <c r="D716" t="n">
+        <v>31</v>
+      </c>
+      <c r="E716" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust api endpoint validation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E716"/>
+  <dimension ref="A1:E717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14029,20 +14029,39 @@
     </row>
     <row r="716">
       <c r="A716" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>31</v>
+      </c>
+      <c r="D716" t="n">
+        <v>31</v>
+      </c>
+      <c r="E716" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B716" t="inlineStr">
+      <c r="B717" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C716" t="n">
-        <v>31</v>
-      </c>
-      <c r="D716" t="n">
-        <v>31</v>
-      </c>
-      <c r="E716" t="n">
+      <c r="C717" t="n">
+        <v>31</v>
+      </c>
+      <c r="D717" t="n">
+        <v>31</v>
+      </c>
+      <c r="E717" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14057,7 +14076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E716"/>
+  <dimension ref="A1:E717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27655,20 +27674,39 @@
     </row>
     <row r="716">
       <c r="A716" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>31</v>
+      </c>
+      <c r="D716" t="n">
+        <v>31</v>
+      </c>
+      <c r="E716" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B716" t="inlineStr">
+      <c r="B717" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C716" t="n">
-        <v>31</v>
-      </c>
-      <c r="D716" t="n">
-        <v>31</v>
-      </c>
-      <c r="E716" t="n">
+      <c r="C717" t="n">
+        <v>31</v>
+      </c>
+      <c r="D717" t="n">
+        <v>31</v>
+      </c>
+      <c r="E717" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E717"/>
+  <dimension ref="A1:E718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14048,20 +14048,39 @@
     </row>
     <row r="717">
       <c r="A717" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>31</v>
+      </c>
+      <c r="D717" t="n">
+        <v>31</v>
+      </c>
+      <c r="E717" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B717" t="inlineStr">
+      <c r="B718" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C717" t="n">
-        <v>31</v>
-      </c>
-      <c r="D717" t="n">
-        <v>31</v>
-      </c>
-      <c r="E717" t="n">
+      <c r="C718" t="n">
+        <v>31</v>
+      </c>
+      <c r="D718" t="n">
+        <v>31</v>
+      </c>
+      <c r="E718" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14076,7 +14095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E717"/>
+  <dimension ref="A1:E718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27693,20 +27712,39 @@
     </row>
     <row r="717">
       <c r="A717" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>31</v>
+      </c>
+      <c r="D717" t="n">
+        <v>31</v>
+      </c>
+      <c r="E717" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B717" t="inlineStr">
+      <c r="B718" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C717" t="n">
-        <v>31</v>
-      </c>
-      <c r="D717" t="n">
-        <v>31</v>
-      </c>
-      <c r="E717" t="n">
+      <c r="C718" t="n">
+        <v>31</v>
+      </c>
+      <c r="D718" t="n">
+        <v>31</v>
+      </c>
+      <c r="E718" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E720"/>
+  <dimension ref="A1:E721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14105,20 +14105,39 @@
     </row>
     <row r="720">
       <c r="A720" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>31</v>
+      </c>
+      <c r="D720" t="n">
+        <v>31</v>
+      </c>
+      <c r="E720" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B720" t="inlineStr">
+      <c r="B721" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C720" t="n">
-        <v>31</v>
-      </c>
-      <c r="D720" t="n">
-        <v>31</v>
-      </c>
-      <c r="E720" t="n">
+      <c r="C721" t="n">
+        <v>31</v>
+      </c>
+      <c r="D721" t="n">
+        <v>31</v>
+      </c>
+      <c r="E721" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14133,7 +14152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E720"/>
+  <dimension ref="A1:E721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27807,20 +27826,39 @@
     </row>
     <row r="720">
       <c r="A720" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>31</v>
+      </c>
+      <c r="D720" t="n">
+        <v>31</v>
+      </c>
+      <c r="E720" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B720" t="inlineStr">
+      <c r="B721" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C720" t="n">
-        <v>31</v>
-      </c>
-      <c r="D720" t="n">
-        <v>31</v>
-      </c>
-      <c r="E720" t="n">
+      <c r="C721" t="n">
+        <v>31</v>
+      </c>
+      <c r="D721" t="n">
+        <v>31</v>
+      </c>
+      <c r="E721" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement error message display
Add input validation for better security.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E721"/>
+  <dimension ref="A1:E722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14124,20 +14124,39 @@
     </row>
     <row r="721">
       <c r="A721" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>31</v>
+      </c>
+      <c r="D721" t="n">
+        <v>31</v>
+      </c>
+      <c r="E721" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B721" t="inlineStr">
+      <c r="B722" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C721" t="n">
-        <v>31</v>
-      </c>
-      <c r="D721" t="n">
-        <v>31</v>
-      </c>
-      <c r="E721" t="n">
+      <c r="C722" t="n">
+        <v>31</v>
+      </c>
+      <c r="D722" t="n">
+        <v>31</v>
+      </c>
+      <c r="E722" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14152,7 +14171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E721"/>
+  <dimension ref="A1:E722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27845,20 +27864,39 @@
     </row>
     <row r="721">
       <c r="A721" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C721" t="n">
+        <v>31</v>
+      </c>
+      <c r="D721" t="n">
+        <v>31</v>
+      </c>
+      <c r="E721" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B721" t="inlineStr">
+      <c r="B722" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C721" t="n">
-        <v>31</v>
-      </c>
-      <c r="D721" t="n">
-        <v>31</v>
-      </c>
-      <c r="E721" t="n">
+      <c r="C722" t="n">
+        <v>31</v>
+      </c>
+      <c r="D722" t="n">
+        <v>31</v>
+      </c>
+      <c r="E722" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E722"/>
+  <dimension ref="A1:E723"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14143,20 +14143,39 @@
     </row>
     <row r="722">
       <c r="A722" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>31</v>
+      </c>
+      <c r="D722" t="n">
+        <v>31</v>
+      </c>
+      <c r="E722" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B722" t="inlineStr">
+      <c r="B723" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C722" t="n">
-        <v>31</v>
-      </c>
-      <c r="D722" t="n">
-        <v>31</v>
-      </c>
-      <c r="E722" t="n">
+      <c r="C723" t="n">
+        <v>31</v>
+      </c>
+      <c r="D723" t="n">
+        <v>31</v>
+      </c>
+      <c r="E723" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14171,7 +14190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E722"/>
+  <dimension ref="A1:E723"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27883,20 +27902,39 @@
     </row>
     <row r="722">
       <c r="A722" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>31</v>
+      </c>
+      <c r="D722" t="n">
+        <v>31</v>
+      </c>
+      <c r="E722" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B722" t="inlineStr">
+      <c r="B723" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C722" t="n">
-        <v>31</v>
-      </c>
-      <c r="D722" t="n">
-        <v>31</v>
-      </c>
-      <c r="E722" t="n">
+      <c r="C723" t="n">
+        <v>31</v>
+      </c>
+      <c r="D723" t="n">
+        <v>31</v>
+      </c>
+      <c r="E723" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E723"/>
+  <dimension ref="A1:E724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14162,20 +14162,39 @@
     </row>
     <row r="723">
       <c r="A723" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>31</v>
+      </c>
+      <c r="D723" t="n">
+        <v>31</v>
+      </c>
+      <c r="E723" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B723" t="inlineStr">
+      <c r="B724" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C723" t="n">
-        <v>31</v>
-      </c>
-      <c r="D723" t="n">
-        <v>31</v>
-      </c>
-      <c r="E723" t="n">
+      <c r="C724" t="n">
+        <v>31</v>
+      </c>
+      <c r="D724" t="n">
+        <v>31</v>
+      </c>
+      <c r="E724" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14190,7 +14209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E723"/>
+  <dimension ref="A1:E724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27921,20 +27940,39 @@
     </row>
     <row r="723">
       <c r="A723" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>31</v>
+      </c>
+      <c r="D723" t="n">
+        <v>31</v>
+      </c>
+      <c r="E723" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B723" t="inlineStr">
+      <c r="B724" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C723" t="n">
-        <v>31</v>
-      </c>
-      <c r="D723" t="n">
-        <v>31</v>
-      </c>
-      <c r="E723" t="n">
+      <c r="C724" t="n">
+        <v>31</v>
+      </c>
+      <c r="D724" t="n">
+        <v>31</v>
+      </c>
+      <c r="E724" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust user authentication module
Improve performance by optimizing database queries.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E724"/>
+  <dimension ref="A1:E725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14181,20 +14181,39 @@
     </row>
     <row r="724">
       <c r="A724" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>31</v>
+      </c>
+      <c r="D724" t="n">
+        <v>31</v>
+      </c>
+      <c r="E724" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B724" t="inlineStr">
+      <c r="B725" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C724" t="n">
-        <v>31</v>
-      </c>
-      <c r="D724" t="n">
-        <v>31</v>
-      </c>
-      <c r="E724" t="n">
+      <c r="C725" t="n">
+        <v>31</v>
+      </c>
+      <c r="D725" t="n">
+        <v>31</v>
+      </c>
+      <c r="E725" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14209,7 +14228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E724"/>
+  <dimension ref="A1:E725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27959,20 +27978,39 @@
     </row>
     <row r="724">
       <c r="A724" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>31</v>
+      </c>
+      <c r="D724" t="n">
+        <v>31</v>
+      </c>
+      <c r="E724" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B724" t="inlineStr">
+      <c r="B725" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C724" t="n">
-        <v>31</v>
-      </c>
-      <c r="D724" t="n">
-        <v>31</v>
-      </c>
-      <c r="E724" t="n">
+      <c r="C725" t="n">
+        <v>31</v>
+      </c>
+      <c r="D725" t="n">
+        <v>31</v>
+      </c>
+      <c r="E725" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize navigation menu accessibility
Update dependencies to their latest versions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E725"/>
+  <dimension ref="A1:E726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14200,20 +14200,39 @@
     </row>
     <row r="725">
       <c r="A725" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>31</v>
+      </c>
+      <c r="D725" t="n">
+        <v>31</v>
+      </c>
+      <c r="E725" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B725" t="inlineStr">
+      <c r="B726" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C725" t="n">
-        <v>31</v>
-      </c>
-      <c r="D725" t="n">
-        <v>31</v>
-      </c>
-      <c r="E725" t="n">
+      <c r="C726" t="n">
+        <v>31</v>
+      </c>
+      <c r="D726" t="n">
+        <v>31</v>
+      </c>
+      <c r="E726" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14228,7 +14247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E725"/>
+  <dimension ref="A1:E726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27997,20 +28016,39 @@
     </row>
     <row r="725">
       <c r="A725" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>31</v>
+      </c>
+      <c r="D725" t="n">
+        <v>31</v>
+      </c>
+      <c r="E725" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B725" t="inlineStr">
+      <c r="B726" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C725" t="n">
-        <v>31</v>
-      </c>
-      <c r="D725" t="n">
-        <v>31</v>
-      </c>
-      <c r="E725" t="n">
+      <c r="C726" t="n">
+        <v>31</v>
+      </c>
+      <c r="D726" t="n">
+        <v>31</v>
+      </c>
+      <c r="E726" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add config file handling
Enhance test coverage to prevent regressions.
Correct null value handling in data processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E726"/>
+  <dimension ref="A1:E727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14219,20 +14219,39 @@
     </row>
     <row r="726">
       <c r="A726" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>31</v>
+      </c>
+      <c r="D726" t="n">
+        <v>31</v>
+      </c>
+      <c r="E726" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B726" t="inlineStr">
+      <c r="B727" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C726" t="n">
-        <v>31</v>
-      </c>
-      <c r="D726" t="n">
-        <v>31</v>
-      </c>
-      <c r="E726" t="n">
+      <c r="C727" t="n">
+        <v>31</v>
+      </c>
+      <c r="D727" t="n">
+        <v>31</v>
+      </c>
+      <c r="E727" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14247,7 +14266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E726"/>
+  <dimension ref="A1:E727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28035,20 +28054,39 @@
     </row>
     <row r="726">
       <c r="A726" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>31</v>
+      </c>
+      <c r="D726" t="n">
+        <v>31</v>
+      </c>
+      <c r="E726" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B726" t="inlineStr">
+      <c r="B727" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C726" t="n">
-        <v>31</v>
-      </c>
-      <c r="D726" t="n">
-        <v>31</v>
-      </c>
-      <c r="E726" t="n">
+      <c r="C727" t="n">
+        <v>31</v>
+      </c>
+      <c r="D727" t="n">
+        <v>31</v>
+      </c>
+      <c r="E727" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E727"/>
+  <dimension ref="A1:E728"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14238,20 +14238,39 @@
     </row>
     <row r="727">
       <c r="A727" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>31</v>
+      </c>
+      <c r="D727" t="n">
+        <v>31</v>
+      </c>
+      <c r="E727" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B727" t="inlineStr">
+      <c r="B728" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C727" t="n">
-        <v>31</v>
-      </c>
-      <c r="D727" t="n">
-        <v>31</v>
-      </c>
-      <c r="E727" t="n">
+      <c r="C728" t="n">
+        <v>31</v>
+      </c>
+      <c r="D728" t="n">
+        <v>31</v>
+      </c>
+      <c r="E728" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14266,7 +14285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E727"/>
+  <dimension ref="A1:E728"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28073,20 +28092,39 @@
     </row>
     <row r="727">
       <c r="A727" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>31</v>
+      </c>
+      <c r="D727" t="n">
+        <v>31</v>
+      </c>
+      <c r="E727" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B727" t="inlineStr">
+      <c r="B728" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C727" t="n">
-        <v>31</v>
-      </c>
-      <c r="D727" t="n">
-        <v>31</v>
-      </c>
-      <c r="E727" t="n">
+      <c r="C728" t="n">
+        <v>31</v>
+      </c>
+      <c r="D728" t="n">
+        <v>31</v>
+      </c>
+      <c r="E728" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Upgrade config file handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E728"/>
+  <dimension ref="A1:E729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14257,20 +14257,39 @@
     </row>
     <row r="728">
       <c r="A728" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>31</v>
+      </c>
+      <c r="D728" t="n">
+        <v>31</v>
+      </c>
+      <c r="E728" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B728" t="inlineStr">
+      <c r="B729" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C728" t="n">
-        <v>31</v>
-      </c>
-      <c r="D728" t="n">
-        <v>31</v>
-      </c>
-      <c r="E728" t="n">
+      <c r="C729" t="n">
+        <v>31</v>
+      </c>
+      <c r="D729" t="n">
+        <v>31</v>
+      </c>
+      <c r="E729" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14285,7 +14304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E728"/>
+  <dimension ref="A1:E729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28111,20 +28130,39 @@
     </row>
     <row r="728">
       <c r="A728" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>31</v>
+      </c>
+      <c r="D728" t="n">
+        <v>31</v>
+      </c>
+      <c r="E728" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B728" t="inlineStr">
+      <c r="B729" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C728" t="n">
-        <v>31</v>
-      </c>
-      <c r="D728" t="n">
-        <v>31</v>
-      </c>
-      <c r="E728" t="n">
+      <c r="C729" t="n">
+        <v>31</v>
+      </c>
+      <c r="D729" t="n">
+        <v>31</v>
+      </c>
+      <c r="E729" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify api endpoint validation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E729"/>
+  <dimension ref="A1:E730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14276,20 +14276,39 @@
     </row>
     <row r="729">
       <c r="A729" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>31</v>
+      </c>
+      <c r="D729" t="n">
+        <v>31</v>
+      </c>
+      <c r="E729" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B729" t="inlineStr">
+      <c r="B730" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C729" t="n">
-        <v>31</v>
-      </c>
-      <c r="D729" t="n">
-        <v>31</v>
-      </c>
-      <c r="E729" t="n">
+      <c r="C730" t="n">
+        <v>31</v>
+      </c>
+      <c r="D730" t="n">
+        <v>31</v>
+      </c>
+      <c r="E730" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14304,7 +14323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E729"/>
+  <dimension ref="A1:E730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28149,20 +28168,39 @@
     </row>
     <row r="729">
       <c r="A729" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>31</v>
+      </c>
+      <c r="D729" t="n">
+        <v>31</v>
+      </c>
+      <c r="E729" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B729" t="inlineStr">
+      <c r="B730" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C729" t="n">
-        <v>31</v>
-      </c>
-      <c r="D729" t="n">
-        <v>31</v>
-      </c>
-      <c r="E729" t="n">
+      <c r="C730" t="n">
+        <v>31</v>
+      </c>
+      <c r="D730" t="n">
+        <v>31</v>
+      </c>
+      <c r="E730" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E730"/>
+  <dimension ref="A1:E731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14295,20 +14295,39 @@
     </row>
     <row r="730">
       <c r="A730" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>31</v>
+      </c>
+      <c r="D730" t="n">
+        <v>31</v>
+      </c>
+      <c r="E730" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B730" t="inlineStr">
+      <c r="B731" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C730" t="n">
-        <v>31</v>
-      </c>
-      <c r="D730" t="n">
-        <v>31</v>
-      </c>
-      <c r="E730" t="n">
+      <c r="C731" t="n">
+        <v>31</v>
+      </c>
+      <c r="D731" t="n">
+        <v>31</v>
+      </c>
+      <c r="E731" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14323,7 +14342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E730"/>
+  <dimension ref="A1:E731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28187,20 +28206,39 @@
     </row>
     <row r="730">
       <c r="A730" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>31</v>
+      </c>
+      <c r="D730" t="n">
+        <v>31</v>
+      </c>
+      <c r="E730" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B730" t="inlineStr">
+      <c r="B731" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C730" t="n">
-        <v>31</v>
-      </c>
-      <c r="D730" t="n">
-        <v>31</v>
-      </c>
-      <c r="E730" t="n">
+      <c r="C731" t="n">
+        <v>31</v>
+      </c>
+      <c r="D731" t="n">
+        <v>31</v>
+      </c>
+      <c r="E731" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E731"/>
+  <dimension ref="A1:E732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14314,20 +14314,39 @@
     </row>
     <row r="731">
       <c r="A731" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>31</v>
+      </c>
+      <c r="D731" t="n">
+        <v>31</v>
+      </c>
+      <c r="E731" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B731" t="inlineStr">
+      <c r="B732" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C731" t="n">
-        <v>31</v>
-      </c>
-      <c r="D731" t="n">
-        <v>31</v>
-      </c>
-      <c r="E731" t="n">
+      <c r="C732" t="n">
+        <v>31</v>
+      </c>
+      <c r="D732" t="n">
+        <v>31</v>
+      </c>
+      <c r="E732" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14342,7 +14361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E731"/>
+  <dimension ref="A1:E732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28225,20 +28244,39 @@
     </row>
     <row r="731">
       <c r="A731" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>31</v>
+      </c>
+      <c r="D731" t="n">
+        <v>31</v>
+      </c>
+      <c r="E731" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B731" t="inlineStr">
+      <c r="B732" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C731" t="n">
-        <v>31</v>
-      </c>
-      <c r="D731" t="n">
-        <v>31</v>
-      </c>
-      <c r="E731" t="n">
+      <c r="C732" t="n">
+        <v>31</v>
+      </c>
+      <c r="D732" t="n">
+        <v>31</v>
+      </c>
+      <c r="E732" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update unit test coverage
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E732"/>
+  <dimension ref="A1:E733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14333,20 +14333,39 @@
     </row>
     <row r="732">
       <c r="A732" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>31</v>
+      </c>
+      <c r="D732" t="n">
+        <v>31</v>
+      </c>
+      <c r="E732" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B732" t="inlineStr">
+      <c r="B733" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C732" t="n">
-        <v>31</v>
-      </c>
-      <c r="D732" t="n">
-        <v>31</v>
-      </c>
-      <c r="E732" t="n">
+      <c r="C733" t="n">
+        <v>31</v>
+      </c>
+      <c r="D733" t="n">
+        <v>31</v>
+      </c>
+      <c r="E733" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14361,7 +14380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E732"/>
+  <dimension ref="A1:E733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28263,20 +28282,39 @@
     </row>
     <row r="732">
       <c r="A732" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>31</v>
+      </c>
+      <c r="D732" t="n">
+        <v>31</v>
+      </c>
+      <c r="E732" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B732" t="inlineStr">
+      <c r="B733" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C732" t="n">
-        <v>31</v>
-      </c>
-      <c r="D732" t="n">
-        <v>31</v>
-      </c>
-      <c r="E732" t="n">
+      <c r="C733" t="n">
+        <v>31</v>
+      </c>
+      <c r="D733" t="n">
+        <v>31</v>
+      </c>
+      <c r="E733" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve user authentication module
Update dependencies to their latest versions.
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E733"/>
+  <dimension ref="A1:E734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14352,20 +14352,39 @@
     </row>
     <row r="733">
       <c r="A733" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>31</v>
+      </c>
+      <c r="D733" t="n">
+        <v>31</v>
+      </c>
+      <c r="E733" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B733" t="inlineStr">
+      <c r="B734" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C733" t="n">
-        <v>31</v>
-      </c>
-      <c r="D733" t="n">
-        <v>31</v>
-      </c>
-      <c r="E733" t="n">
+      <c r="C734" t="n">
+        <v>31</v>
+      </c>
+      <c r="D734" t="n">
+        <v>31</v>
+      </c>
+      <c r="E734" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14380,7 +14399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E733"/>
+  <dimension ref="A1:E734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28301,20 +28320,39 @@
     </row>
     <row r="733">
       <c r="A733" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>31</v>
+      </c>
+      <c r="D733" t="n">
+        <v>31</v>
+      </c>
+      <c r="E733" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B733" t="inlineStr">
+      <c r="B734" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C733" t="n">
-        <v>31</v>
-      </c>
-      <c r="D733" t="n">
-        <v>31</v>
-      </c>
-      <c r="E733" t="n">
+      <c r="C734" t="n">
+        <v>31</v>
+      </c>
+      <c r="D734" t="n">
+        <v>31</v>
+      </c>
+      <c r="E734" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update navigation menu accessibility
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E735"/>
+  <dimension ref="A1:E736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14390,20 +14390,39 @@
     </row>
     <row r="735">
       <c r="A735" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>31</v>
+      </c>
+      <c r="D735" t="n">
+        <v>31</v>
+      </c>
+      <c r="E735" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B735" t="inlineStr">
+      <c r="B736" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C735" t="n">
-        <v>31</v>
-      </c>
-      <c r="D735" t="n">
-        <v>31</v>
-      </c>
-      <c r="E735" t="n">
+      <c r="C736" t="n">
+        <v>31</v>
+      </c>
+      <c r="D736" t="n">
+        <v>31</v>
+      </c>
+      <c r="E736" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14418,7 +14437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E735"/>
+  <dimension ref="A1:E736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28377,20 +28396,39 @@
     </row>
     <row r="735">
       <c r="A735" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>31</v>
+      </c>
+      <c r="D735" t="n">
+        <v>31</v>
+      </c>
+      <c r="E735" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B735" t="inlineStr">
+      <c r="B736" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C735" t="n">
-        <v>31</v>
-      </c>
-      <c r="D735" t="n">
-        <v>31</v>
-      </c>
-      <c r="E735" t="n">
+      <c r="C736" t="n">
+        <v>31</v>
+      </c>
+      <c r="D736" t="n">
+        <v>31</v>
+      </c>
+      <c r="E736" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise config file handling
Correct null value handling in data processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E736"/>
+  <dimension ref="A1:E737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14409,20 +14409,39 @@
     </row>
     <row r="736">
       <c r="A736" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>31</v>
+      </c>
+      <c r="D736" t="n">
+        <v>31</v>
+      </c>
+      <c r="E736" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B736" t="inlineStr">
+      <c r="B737" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C736" t="n">
-        <v>31</v>
-      </c>
-      <c r="D736" t="n">
-        <v>31</v>
-      </c>
-      <c r="E736" t="n">
+      <c r="C737" t="n">
+        <v>31</v>
+      </c>
+      <c r="D737" t="n">
+        <v>31</v>
+      </c>
+      <c r="E737" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14437,7 +14456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E736"/>
+  <dimension ref="A1:E737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28415,20 +28434,39 @@
     </row>
     <row r="736">
       <c r="A736" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>31</v>
+      </c>
+      <c r="D736" t="n">
+        <v>31</v>
+      </c>
+      <c r="E736" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B736" t="inlineStr">
+      <c r="B737" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C736" t="n">
-        <v>31</v>
-      </c>
-      <c r="D736" t="n">
-        <v>31</v>
-      </c>
-      <c r="E736" t="n">
+      <c r="C737" t="n">
+        <v>31</v>
+      </c>
+      <c r="D737" t="n">
+        <v>31</v>
+      </c>
+      <c r="E737" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove api response formatting
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E740"/>
+  <dimension ref="A1:E741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14485,20 +14485,39 @@
     </row>
     <row r="740">
       <c r="A740" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>31</v>
+      </c>
+      <c r="D740" t="n">
+        <v>31</v>
+      </c>
+      <c r="E740" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B740" t="inlineStr">
+      <c r="B741" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C740" t="n">
-        <v>31</v>
-      </c>
-      <c r="D740" t="n">
-        <v>31</v>
-      </c>
-      <c r="E740" t="n">
+      <c r="C741" t="n">
+        <v>31</v>
+      </c>
+      <c r="D741" t="n">
+        <v>31</v>
+      </c>
+      <c r="E741" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14513,7 +14532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E740"/>
+  <dimension ref="A1:E741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28567,20 +28586,39 @@
     </row>
     <row r="740">
       <c r="A740" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>31</v>
+      </c>
+      <c r="D740" t="n">
+        <v>31</v>
+      </c>
+      <c r="E740" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B740" t="inlineStr">
+      <c r="B741" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C740" t="n">
-        <v>31</v>
-      </c>
-      <c r="D740" t="n">
-        <v>31</v>
-      </c>
-      <c r="E740" t="n">
+      <c r="C741" t="n">
+        <v>31</v>
+      </c>
+      <c r="D741" t="n">
+        <v>31</v>
+      </c>
+      <c r="E741" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize error message display
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E741"/>
+  <dimension ref="A1:E742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14504,20 +14504,39 @@
     </row>
     <row r="741">
       <c r="A741" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>31</v>
+      </c>
+      <c r="D741" t="n">
+        <v>31</v>
+      </c>
+      <c r="E741" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B741" t="inlineStr">
+      <c r="B742" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C741" t="n">
-        <v>31</v>
-      </c>
-      <c r="D741" t="n">
-        <v>31</v>
-      </c>
-      <c r="E741" t="n">
+      <c r="C742" t="n">
+        <v>31</v>
+      </c>
+      <c r="D742" t="n">
+        <v>31</v>
+      </c>
+      <c r="E742" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14532,7 +14551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E741"/>
+  <dimension ref="A1:E742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28605,20 +28624,39 @@
     </row>
     <row r="741">
       <c r="A741" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>31</v>
+      </c>
+      <c r="D741" t="n">
+        <v>31</v>
+      </c>
+      <c r="E741" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B741" t="inlineStr">
+      <c r="B742" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C741" t="n">
-        <v>31</v>
-      </c>
-      <c r="D741" t="n">
-        <v>31</v>
-      </c>
-      <c r="E741" t="n">
+      <c r="C742" t="n">
+        <v>31</v>
+      </c>
+      <c r="D742" t="n">
+        <v>31</v>
+      </c>
+      <c r="E742" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise build script optimization
Remove deprecated functions and clean up codebase.
Improve performance by optimizing database queries.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E742"/>
+  <dimension ref="A1:E743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14523,20 +14523,39 @@
     </row>
     <row r="742">
       <c r="A742" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>31</v>
+      </c>
+      <c r="D742" t="n">
+        <v>31</v>
+      </c>
+      <c r="E742" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B742" t="inlineStr">
+      <c r="B743" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C742" t="n">
-        <v>31</v>
-      </c>
-      <c r="D742" t="n">
-        <v>31</v>
-      </c>
-      <c r="E742" t="n">
+      <c r="C743" t="n">
+        <v>31</v>
+      </c>
+      <c r="D743" t="n">
+        <v>31</v>
+      </c>
+      <c r="E743" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14551,7 +14570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E742"/>
+  <dimension ref="A1:E743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28643,20 +28662,39 @@
     </row>
     <row r="742">
       <c r="A742" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>31</v>
+      </c>
+      <c r="D742" t="n">
+        <v>31</v>
+      </c>
+      <c r="E742" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B742" t="inlineStr">
+      <c r="B743" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C742" t="n">
-        <v>31</v>
-      </c>
-      <c r="D742" t="n">
-        <v>31</v>
-      </c>
-      <c r="E742" t="n">
+      <c r="C743" t="n">
+        <v>31</v>
+      </c>
+      <c r="D743" t="n">
+        <v>31</v>
+      </c>
+      <c r="E743" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove navigation menu accessibility
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E743"/>
+  <dimension ref="A1:E744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14542,20 +14542,39 @@
     </row>
     <row r="743">
       <c r="A743" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>31</v>
+      </c>
+      <c r="D743" t="n">
+        <v>31</v>
+      </c>
+      <c r="E743" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B743" t="inlineStr">
+      <c r="B744" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C743" t="n">
-        <v>31</v>
-      </c>
-      <c r="D743" t="n">
-        <v>31</v>
-      </c>
-      <c r="E743" t="n">
+      <c r="C744" t="n">
+        <v>31</v>
+      </c>
+      <c r="D744" t="n">
+        <v>31</v>
+      </c>
+      <c r="E744" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14570,7 +14589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E743"/>
+  <dimension ref="A1:E744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28681,20 +28700,39 @@
     </row>
     <row r="743">
       <c r="A743" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>31</v>
+      </c>
+      <c r="D743" t="n">
+        <v>31</v>
+      </c>
+      <c r="E743" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B743" t="inlineStr">
+      <c r="B744" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C743" t="n">
-        <v>31</v>
-      </c>
-      <c r="D743" t="n">
-        <v>31</v>
-      </c>
-      <c r="E743" t="n">
+      <c r="C744" t="n">
+        <v>31</v>
+      </c>
+      <c r="D744" t="n">
+        <v>31</v>
+      </c>
+      <c r="E744" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise api endpoint validation
This resolves issue #12.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E745"/>
+  <dimension ref="A1:E746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14580,20 +14580,39 @@
     </row>
     <row r="745">
       <c r="A745" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>31</v>
+      </c>
+      <c r="D745" t="n">
+        <v>31</v>
+      </c>
+      <c r="E745" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B745" t="inlineStr">
+      <c r="B746" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C745" t="n">
-        <v>31</v>
-      </c>
-      <c r="D745" t="n">
-        <v>31</v>
-      </c>
-      <c r="E745" t="n">
+      <c r="C746" t="n">
+        <v>31</v>
+      </c>
+      <c r="D746" t="n">
+        <v>31</v>
+      </c>
+      <c r="E746" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14608,7 +14627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E745"/>
+  <dimension ref="A1:E746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28757,20 +28776,39 @@
     </row>
     <row r="745">
       <c r="A745" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>31</v>
+      </c>
+      <c r="D745" t="n">
+        <v>31</v>
+      </c>
+      <c r="E745" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B745" t="inlineStr">
+      <c r="B746" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C745" t="n">
-        <v>31</v>
-      </c>
-      <c r="D745" t="n">
-        <v>31</v>
-      </c>
-      <c r="E745" t="n">
+      <c r="C746" t="n">
+        <v>31</v>
+      </c>
+      <c r="D746" t="n">
+        <v>31</v>
+      </c>
+      <c r="E746" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove login page ui elements
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E749"/>
+  <dimension ref="A1:E750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14656,20 +14656,39 @@
     </row>
     <row r="749">
       <c r="A749" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C749" t="n">
+        <v>31</v>
+      </c>
+      <c r="D749" t="n">
+        <v>31</v>
+      </c>
+      <c r="E749" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B749" t="inlineStr">
+      <c r="B750" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C749" t="n">
-        <v>31</v>
-      </c>
-      <c r="D749" t="n">
-        <v>31</v>
-      </c>
-      <c r="E749" t="n">
+      <c r="C750" t="n">
+        <v>31</v>
+      </c>
+      <c r="D750" t="n">
+        <v>31</v>
+      </c>
+      <c r="E750" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14684,7 +14703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E749"/>
+  <dimension ref="A1:E750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28909,20 +28928,39 @@
     </row>
     <row r="749">
       <c r="A749" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C749" t="n">
+        <v>31</v>
+      </c>
+      <c r="D749" t="n">
+        <v>31</v>
+      </c>
+      <c r="E749" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B749" t="inlineStr">
+      <c r="B750" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C749" t="n">
-        <v>31</v>
-      </c>
-      <c r="D749" t="n">
-        <v>31</v>
-      </c>
-      <c r="E749" t="n">
+      <c r="C750" t="n">
+        <v>31</v>
+      </c>
+      <c r="D750" t="n">
+        <v>31</v>
+      </c>
+      <c r="E750" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct api endpoint validation
Correct null value handling in data processing.
Refactor legacy code to follow modern practices.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E752"/>
+  <dimension ref="A1:E753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14713,20 +14713,39 @@
     </row>
     <row r="752">
       <c r="A752" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C752" t="n">
+        <v>31</v>
+      </c>
+      <c r="D752" t="n">
+        <v>31</v>
+      </c>
+      <c r="E752" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B752" t="inlineStr">
+      <c r="B753" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C752" t="n">
-        <v>31</v>
-      </c>
-      <c r="D752" t="n">
-        <v>31</v>
-      </c>
-      <c r="E752" t="n">
+      <c r="C753" t="n">
+        <v>31</v>
+      </c>
+      <c r="D753" t="n">
+        <v>31</v>
+      </c>
+      <c r="E753" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14741,7 +14760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E752"/>
+  <dimension ref="A1:E753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29023,20 +29042,39 @@
     </row>
     <row r="752">
       <c r="A752" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C752" t="n">
+        <v>31</v>
+      </c>
+      <c r="D752" t="n">
+        <v>31</v>
+      </c>
+      <c r="E752" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B752" t="inlineStr">
+      <c r="B753" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C752" t="n">
-        <v>31</v>
-      </c>
-      <c r="D752" t="n">
-        <v>31</v>
-      </c>
-      <c r="E752" t="n">
+      <c r="C753" t="n">
+        <v>31</v>
+      </c>
+      <c r="D753" t="n">
+        <v>31</v>
+      </c>
+      <c r="E753" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add responsive design implementation
Correct null value handling in data processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E753"/>
+  <dimension ref="A1:E754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14732,20 +14732,39 @@
     </row>
     <row r="753">
       <c r="A753" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C753" t="n">
+        <v>31</v>
+      </c>
+      <c r="D753" t="n">
+        <v>31</v>
+      </c>
+      <c r="E753" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B753" t="inlineStr">
+      <c r="B754" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C753" t="n">
-        <v>31</v>
-      </c>
-      <c r="D753" t="n">
-        <v>31</v>
-      </c>
-      <c r="E753" t="n">
+      <c r="C754" t="n">
+        <v>31</v>
+      </c>
+      <c r="D754" t="n">
+        <v>31</v>
+      </c>
+      <c r="E754" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14760,7 +14779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E753"/>
+  <dimension ref="A1:E754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29061,20 +29080,39 @@
     </row>
     <row r="753">
       <c r="A753" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C753" t="n">
+        <v>31</v>
+      </c>
+      <c r="D753" t="n">
+        <v>31</v>
+      </c>
+      <c r="E753" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B753" t="inlineStr">
+      <c r="B754" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C753" t="n">
-        <v>31</v>
-      </c>
-      <c r="D753" t="n">
-        <v>31</v>
-      </c>
-      <c r="E753" t="n">
+      <c r="C754" t="n">
+        <v>31</v>
+      </c>
+      <c r="D754" t="n">
+        <v>31</v>
+      </c>
+      <c r="E754" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove responsive design implementation
Apply code style fixes as per linter recommendations.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E754"/>
+  <dimension ref="A1:E755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14751,20 +14751,39 @@
     </row>
     <row r="754">
       <c r="A754" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>31</v>
+      </c>
+      <c r="D754" t="n">
+        <v>31</v>
+      </c>
+      <c r="E754" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B754" t="inlineStr">
+      <c r="B755" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C754" t="n">
-        <v>31</v>
-      </c>
-      <c r="D754" t="n">
-        <v>31</v>
-      </c>
-      <c r="E754" t="n">
+      <c r="C755" t="n">
+        <v>31</v>
+      </c>
+      <c r="D755" t="n">
+        <v>31</v>
+      </c>
+      <c r="E755" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14779,7 +14798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E754"/>
+  <dimension ref="A1:E755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29099,20 +29118,39 @@
     </row>
     <row r="754">
       <c r="A754" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>31</v>
+      </c>
+      <c r="D754" t="n">
+        <v>31</v>
+      </c>
+      <c r="E754" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B754" t="inlineStr">
+      <c r="B755" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C754" t="n">
-        <v>31</v>
-      </c>
-      <c r="D754" t="n">
-        <v>31</v>
-      </c>
-      <c r="E754" t="n">
+      <c r="C755" t="n">
+        <v>31</v>
+      </c>
+      <c r="D755" t="n">
+        <v>31</v>
+      </c>
+      <c r="E755" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify logging system configuration
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E756"/>
+  <dimension ref="A1:E757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14789,20 +14789,39 @@
     </row>
     <row r="756">
       <c r="A756" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>31</v>
+      </c>
+      <c r="D756" t="n">
+        <v>31</v>
+      </c>
+      <c r="E756" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B756" t="inlineStr">
+      <c r="B757" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C756" t="n">
-        <v>31</v>
-      </c>
-      <c r="D756" t="n">
-        <v>31</v>
-      </c>
-      <c r="E756" t="n">
+      <c r="C757" t="n">
+        <v>31</v>
+      </c>
+      <c r="D757" t="n">
+        <v>31</v>
+      </c>
+      <c r="E757" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14817,7 +14836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E756"/>
+  <dimension ref="A1:E757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29175,20 +29194,39 @@
     </row>
     <row r="756">
       <c r="A756" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>31</v>
+      </c>
+      <c r="D756" t="n">
+        <v>31</v>
+      </c>
+      <c r="E756" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B756" t="inlineStr">
+      <c r="B757" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C756" t="n">
-        <v>31</v>
-      </c>
-      <c r="D756" t="n">
-        <v>31</v>
-      </c>
-      <c r="E756" t="n">
+      <c r="C757" t="n">
+        <v>31</v>
+      </c>
+      <c r="D757" t="n">
+        <v>31</v>
+      </c>
+      <c r="E757" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert file upload functionality
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E757"/>
+  <dimension ref="A1:E758"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14808,20 +14808,39 @@
     </row>
     <row r="757">
       <c r="A757" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>31</v>
+      </c>
+      <c r="D757" t="n">
+        <v>31</v>
+      </c>
+      <c r="E757" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B757" t="inlineStr">
+      <c r="B758" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C757" t="n">
-        <v>31</v>
-      </c>
-      <c r="D757" t="n">
-        <v>31</v>
-      </c>
-      <c r="E757" t="n">
+      <c r="C758" t="n">
+        <v>31</v>
+      </c>
+      <c r="D758" t="n">
+        <v>31</v>
+      </c>
+      <c r="E758" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14836,7 +14855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E757"/>
+  <dimension ref="A1:E758"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29213,20 +29232,39 @@
     </row>
     <row r="757">
       <c r="A757" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>31</v>
+      </c>
+      <c r="D757" t="n">
+        <v>31</v>
+      </c>
+      <c r="E757" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B757" t="inlineStr">
+      <c r="B758" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C757" t="n">
-        <v>31</v>
-      </c>
-      <c r="D757" t="n">
-        <v>31</v>
-      </c>
-      <c r="E757" t="n">
+      <c r="C758" t="n">
+        <v>31</v>
+      </c>
+      <c r="D758" t="n">
+        <v>31</v>
+      </c>
+      <c r="E758" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust logging system configuration
Address edge cases reported in user feedback.
Fix various typos in comments and documentation.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E758"/>
+  <dimension ref="A1:E759"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14827,20 +14827,39 @@
     </row>
     <row r="758">
       <c r="A758" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>31</v>
+      </c>
+      <c r="D758" t="n">
+        <v>31</v>
+      </c>
+      <c r="E758" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B758" t="inlineStr">
+      <c r="B759" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C758" t="n">
-        <v>31</v>
-      </c>
-      <c r="D758" t="n">
-        <v>31</v>
-      </c>
-      <c r="E758" t="n">
+      <c r="C759" t="n">
+        <v>31</v>
+      </c>
+      <c r="D759" t="n">
+        <v>31</v>
+      </c>
+      <c r="E759" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14855,7 +14874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E758"/>
+  <dimension ref="A1:E759"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29251,20 +29270,39 @@
     </row>
     <row r="758">
       <c r="A758" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>31</v>
+      </c>
+      <c r="D758" t="n">
+        <v>31</v>
+      </c>
+      <c r="E758" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B758" t="inlineStr">
+      <c r="B759" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C758" t="n">
-        <v>31</v>
-      </c>
-      <c r="D758" t="n">
-        <v>31</v>
-      </c>
-      <c r="E758" t="n">
+      <c r="C759" t="n">
+        <v>31</v>
+      </c>
+      <c r="D759" t="n">
+        <v>31</v>
+      </c>
+      <c r="E759" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E760"/>
+  <dimension ref="A1:E761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14865,20 +14865,39 @@
     </row>
     <row r="760">
       <c r="A760" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>31</v>
+      </c>
+      <c r="D760" t="n">
+        <v>31</v>
+      </c>
+      <c r="E760" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B760" t="inlineStr">
+      <c r="B761" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C760" t="n">
-        <v>31</v>
-      </c>
-      <c r="D760" t="n">
-        <v>31</v>
-      </c>
-      <c r="E760" t="n">
+      <c r="C761" t="n">
+        <v>31</v>
+      </c>
+      <c r="D761" t="n">
+        <v>31</v>
+      </c>
+      <c r="E761" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14893,7 +14912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E760"/>
+  <dimension ref="A1:E761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29327,20 +29346,39 @@
     </row>
     <row r="760">
       <c r="A760" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>31</v>
+      </c>
+      <c r="D760" t="n">
+        <v>31</v>
+      </c>
+      <c r="E760" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B760" t="inlineStr">
+      <c r="B761" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C760" t="n">
-        <v>31</v>
-      </c>
-      <c r="D760" t="n">
-        <v>31</v>
-      </c>
-      <c r="E760" t="n">
+      <c r="C761" t="n">
+        <v>31</v>
+      </c>
+      <c r="D761" t="n">
+        <v>31</v>
+      </c>
+      <c r="E761" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance logging system configuration
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E761"/>
+  <dimension ref="A1:E762"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14884,20 +14884,39 @@
     </row>
     <row r="761">
       <c r="A761" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>31</v>
+      </c>
+      <c r="D761" t="n">
+        <v>31</v>
+      </c>
+      <c r="E761" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B761" t="inlineStr">
+      <c r="B762" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C761" t="n">
-        <v>31</v>
-      </c>
-      <c r="D761" t="n">
-        <v>31</v>
-      </c>
-      <c r="E761" t="n">
+      <c r="C762" t="n">
+        <v>31</v>
+      </c>
+      <c r="D762" t="n">
+        <v>31</v>
+      </c>
+      <c r="E762" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14912,7 +14931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E761"/>
+  <dimension ref="A1:E762"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29365,20 +29384,39 @@
     </row>
     <row r="761">
       <c r="A761" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>31</v>
+      </c>
+      <c r="D761" t="n">
+        <v>31</v>
+      </c>
+      <c r="E761" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B761" t="inlineStr">
+      <c r="B762" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C761" t="n">
-        <v>31</v>
-      </c>
-      <c r="D761" t="n">
-        <v>31</v>
-      </c>
-      <c r="E761" t="n">
+      <c r="C762" t="n">
+        <v>31</v>
+      </c>
+      <c r="D762" t="n">
+        <v>31</v>
+      </c>
+      <c r="E762" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add image processing memory leaks
Fix various typos in comments and documentation.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E762"/>
+  <dimension ref="A1:E763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14903,20 +14903,39 @@
     </row>
     <row r="762">
       <c r="A762" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C762" t="n">
+        <v>31</v>
+      </c>
+      <c r="D762" t="n">
+        <v>31</v>
+      </c>
+      <c r="E762" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B762" t="inlineStr">
+      <c r="B763" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C762" t="n">
-        <v>31</v>
-      </c>
-      <c r="D762" t="n">
-        <v>31</v>
-      </c>
-      <c r="E762" t="n">
+      <c r="C763" t="n">
+        <v>31</v>
+      </c>
+      <c r="D763" t="n">
+        <v>31</v>
+      </c>
+      <c r="E763" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14931,7 +14950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E762"/>
+  <dimension ref="A1:E763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29403,20 +29422,39 @@
     </row>
     <row r="762">
       <c r="A762" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C762" t="n">
+        <v>31</v>
+      </c>
+      <c r="D762" t="n">
+        <v>31</v>
+      </c>
+      <c r="E762" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B762" t="inlineStr">
+      <c r="B763" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C762" t="n">
-        <v>31</v>
-      </c>
-      <c r="D762" t="n">
-        <v>31</v>
-      </c>
-      <c r="E762" t="n">
+      <c r="C763" t="n">
+        <v>31</v>
+      </c>
+      <c r="D763" t="n">
+        <v>31</v>
+      </c>
+      <c r="E763" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E764"/>
+  <dimension ref="A1:E765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14941,20 +14941,39 @@
     </row>
     <row r="764">
       <c r="A764" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>31</v>
+      </c>
+      <c r="D764" t="n">
+        <v>31</v>
+      </c>
+      <c r="E764" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B764" t="inlineStr">
+      <c r="B765" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C764" t="n">
-        <v>31</v>
-      </c>
-      <c r="D764" t="n">
-        <v>31</v>
-      </c>
-      <c r="E764" t="n">
+      <c r="C765" t="n">
+        <v>31</v>
+      </c>
+      <c r="D765" t="n">
+        <v>31</v>
+      </c>
+      <c r="E765" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14969,7 +14988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E764"/>
+  <dimension ref="A1:E765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29479,20 +29498,39 @@
     </row>
     <row r="764">
       <c r="A764" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>31</v>
+      </c>
+      <c r="D764" t="n">
+        <v>31</v>
+      </c>
+      <c r="E764" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B764" t="inlineStr">
+      <c r="B765" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C764" t="n">
-        <v>31</v>
-      </c>
-      <c r="D764" t="n">
-        <v>31</v>
-      </c>
-      <c r="E764" t="n">
+      <c r="C765" t="n">
+        <v>31</v>
+      </c>
+      <c r="D765" t="n">
+        <v>31</v>
+      </c>
+      <c r="E765" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E765"/>
+  <dimension ref="A1:E766"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14960,20 +14960,39 @@
     </row>
     <row r="765">
       <c r="A765" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>31</v>
+      </c>
+      <c r="D765" t="n">
+        <v>31</v>
+      </c>
+      <c r="E765" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B765" t="inlineStr">
+      <c r="B766" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C765" t="n">
-        <v>31</v>
-      </c>
-      <c r="D765" t="n">
-        <v>31</v>
-      </c>
-      <c r="E765" t="n">
+      <c r="C766" t="n">
+        <v>31</v>
+      </c>
+      <c r="D766" t="n">
+        <v>31</v>
+      </c>
+      <c r="E766" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14988,7 +15007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E765"/>
+  <dimension ref="A1:E766"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29517,20 +29536,39 @@
     </row>
     <row r="765">
       <c r="A765" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>31</v>
+      </c>
+      <c r="D765" t="n">
+        <v>31</v>
+      </c>
+      <c r="E765" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B765" t="inlineStr">
+      <c r="B766" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C765" t="n">
-        <v>31</v>
-      </c>
-      <c r="D765" t="n">
-        <v>31</v>
-      </c>
-      <c r="E765" t="n">
+      <c r="C766" t="n">
+        <v>31</v>
+      </c>
+      <c r="D766" t="n">
+        <v>31</v>
+      </c>
+      <c r="E766" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix file upload functionality
Optimize image compression algorithm.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E767"/>
+  <dimension ref="A1:E768"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14998,20 +14998,39 @@
     </row>
     <row r="767">
       <c r="A767" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>31</v>
+      </c>
+      <c r="D767" t="n">
+        <v>31</v>
+      </c>
+      <c r="E767" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B767" t="inlineStr">
+      <c r="B768" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C767" t="n">
-        <v>31</v>
-      </c>
-      <c r="D767" t="n">
-        <v>31</v>
-      </c>
-      <c r="E767" t="n">
+      <c r="C768" t="n">
+        <v>31</v>
+      </c>
+      <c r="D768" t="n">
+        <v>31</v>
+      </c>
+      <c r="E768" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15026,7 +15045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E767"/>
+  <dimension ref="A1:E768"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29593,20 +29612,39 @@
     </row>
     <row r="767">
       <c r="A767" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>31</v>
+      </c>
+      <c r="D767" t="n">
+        <v>31</v>
+      </c>
+      <c r="E767" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B767" t="inlineStr">
+      <c r="B768" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C767" t="n">
-        <v>31</v>
-      </c>
-      <c r="D767" t="n">
-        <v>31</v>
-      </c>
-      <c r="E767" t="n">
+      <c r="C768" t="n">
+        <v>31</v>
+      </c>
+      <c r="D768" t="n">
+        <v>31</v>
+      </c>
+      <c r="E768" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E769"/>
+  <dimension ref="A1:E770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15036,20 +15036,39 @@
     </row>
     <row r="769">
       <c r="A769" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>31</v>
+      </c>
+      <c r="D769" t="n">
+        <v>31</v>
+      </c>
+      <c r="E769" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B769" t="inlineStr">
+      <c r="B770" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C769" t="n">
-        <v>31</v>
-      </c>
-      <c r="D769" t="n">
-        <v>31</v>
-      </c>
-      <c r="E769" t="n">
+      <c r="C770" t="n">
+        <v>31</v>
+      </c>
+      <c r="D770" t="n">
+        <v>31</v>
+      </c>
+      <c r="E770" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15064,7 +15083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E769"/>
+  <dimension ref="A1:E770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29669,20 +29688,39 @@
     </row>
     <row r="769">
       <c r="A769" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>31</v>
+      </c>
+      <c r="D769" t="n">
+        <v>31</v>
+      </c>
+      <c r="E769" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B769" t="inlineStr">
+      <c r="B770" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C769" t="n">
-        <v>31</v>
-      </c>
-      <c r="D769" t="n">
-        <v>31</v>
-      </c>
-      <c r="E769" t="n">
+      <c r="C770" t="n">
+        <v>31</v>
+      </c>
+      <c r="D770" t="n">
+        <v>31</v>
+      </c>
+      <c r="E770" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve database schema migration
Apply code style fixes as per linter recommendations.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E775"/>
+  <dimension ref="A1:E776"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15150,20 +15150,39 @@
     </row>
     <row r="775">
       <c r="A775" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>31</v>
+      </c>
+      <c r="D775" t="n">
+        <v>31</v>
+      </c>
+      <c r="E775" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B775" t="inlineStr">
+      <c r="B776" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C775" t="n">
-        <v>31</v>
-      </c>
-      <c r="D775" t="n">
-        <v>31</v>
-      </c>
-      <c r="E775" t="n">
+      <c r="C776" t="n">
+        <v>31</v>
+      </c>
+      <c r="D776" t="n">
+        <v>31</v>
+      </c>
+      <c r="E776" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15178,7 +15197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E775"/>
+  <dimension ref="A1:E776"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29897,20 +29916,39 @@
     </row>
     <row r="775">
       <c r="A775" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>31</v>
+      </c>
+      <c r="D775" t="n">
+        <v>31</v>
+      </c>
+      <c r="E775" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B775" t="inlineStr">
+      <c r="B776" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C775" t="n">
-        <v>31</v>
-      </c>
-      <c r="D775" t="n">
-        <v>31</v>
-      </c>
-      <c r="E775" t="n">
+      <c r="C776" t="n">
+        <v>31</v>
+      </c>
+      <c r="D776" t="n">
+        <v>31</v>
+      </c>
+      <c r="E776" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize unit test coverage
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E777"/>
+  <dimension ref="A1:E778"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15188,20 +15188,39 @@
     </row>
     <row r="777">
       <c r="A777" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C777" t="n">
+        <v>31</v>
+      </c>
+      <c r="D777" t="n">
+        <v>31</v>
+      </c>
+      <c r="E777" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B777" t="inlineStr">
+      <c r="B778" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C777" t="n">
-        <v>31</v>
-      </c>
-      <c r="D777" t="n">
-        <v>31</v>
-      </c>
-      <c r="E777" t="n">
+      <c r="C778" t="n">
+        <v>31</v>
+      </c>
+      <c r="D778" t="n">
+        <v>31</v>
+      </c>
+      <c r="E778" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15216,7 +15235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E777"/>
+  <dimension ref="A1:E778"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29973,20 +29992,39 @@
     </row>
     <row r="777">
       <c r="A777" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C777" t="n">
+        <v>31</v>
+      </c>
+      <c r="D777" t="n">
+        <v>31</v>
+      </c>
+      <c r="E777" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B777" t="inlineStr">
+      <c r="B778" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C777" t="n">
-        <v>31</v>
-      </c>
-      <c r="D777" t="n">
-        <v>31</v>
-      </c>
-      <c r="E777" t="n">
+      <c r="C778" t="n">
+        <v>31</v>
+      </c>
+      <c r="D778" t="n">
+        <v>31</v>
+      </c>
+      <c r="E778" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E778"/>
+  <dimension ref="A1:E779"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15207,20 +15207,39 @@
     </row>
     <row r="778">
       <c r="A778" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>31</v>
+      </c>
+      <c r="D778" t="n">
+        <v>31</v>
+      </c>
+      <c r="E778" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B778" t="inlineStr">
+      <c r="B779" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C778" t="n">
-        <v>31</v>
-      </c>
-      <c r="D778" t="n">
-        <v>31</v>
-      </c>
-      <c r="E778" t="n">
+      <c r="C779" t="n">
+        <v>31</v>
+      </c>
+      <c r="D779" t="n">
+        <v>31</v>
+      </c>
+      <c r="E779" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15235,7 +15254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E778"/>
+  <dimension ref="A1:E779"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30011,20 +30030,39 @@
     </row>
     <row r="778">
       <c r="A778" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>31</v>
+      </c>
+      <c r="D778" t="n">
+        <v>31</v>
+      </c>
+      <c r="E778" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B778" t="inlineStr">
+      <c r="B779" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C778" t="n">
-        <v>31</v>
-      </c>
-      <c r="D778" t="n">
-        <v>31</v>
-      </c>
-      <c r="E778" t="n">
+      <c r="C779" t="n">
+        <v>31</v>
+      </c>
+      <c r="D779" t="n">
+        <v>31</v>
+      </c>
+      <c r="E779" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E779"/>
+  <dimension ref="A1:E780"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15226,20 +15226,39 @@
     </row>
     <row r="779">
       <c r="A779" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>31</v>
+      </c>
+      <c r="D779" t="n">
+        <v>31</v>
+      </c>
+      <c r="E779" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B779" t="inlineStr">
+      <c r="B780" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C779" t="n">
-        <v>31</v>
-      </c>
-      <c r="D779" t="n">
-        <v>31</v>
-      </c>
-      <c r="E779" t="n">
+      <c r="C780" t="n">
+        <v>31</v>
+      </c>
+      <c r="D780" t="n">
+        <v>31</v>
+      </c>
+      <c r="E780" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15254,7 +15273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E779"/>
+  <dimension ref="A1:E780"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30049,20 +30068,39 @@
     </row>
     <row r="779">
       <c r="A779" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>31</v>
+      </c>
+      <c r="D779" t="n">
+        <v>31</v>
+      </c>
+      <c r="E779" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B779" t="inlineStr">
+      <c r="B780" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C779" t="n">
-        <v>31</v>
-      </c>
-      <c r="D779" t="n">
-        <v>31</v>
-      </c>
-      <c r="E779" t="n">
+      <c r="C780" t="n">
+        <v>31</v>
+      </c>
+      <c r="D780" t="n">
+        <v>31</v>
+      </c>
+      <c r="E780" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E780"/>
+  <dimension ref="A1:E781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15245,20 +15245,39 @@
     </row>
     <row r="780">
       <c r="A780" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>31</v>
+      </c>
+      <c r="D780" t="n">
+        <v>31</v>
+      </c>
+      <c r="E780" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B780" t="inlineStr">
+      <c r="B781" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C780" t="n">
-        <v>31</v>
-      </c>
-      <c r="D780" t="n">
-        <v>31</v>
-      </c>
-      <c r="E780" t="n">
+      <c r="C781" t="n">
+        <v>31</v>
+      </c>
+      <c r="D781" t="n">
+        <v>31</v>
+      </c>
+      <c r="E781" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15273,7 +15292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E780"/>
+  <dimension ref="A1:E781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30087,20 +30106,39 @@
     </row>
     <row r="780">
       <c r="A780" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>31</v>
+      </c>
+      <c r="D780" t="n">
+        <v>31</v>
+      </c>
+      <c r="E780" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B780" t="inlineStr">
+      <c r="B781" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C780" t="n">
-        <v>31</v>
-      </c>
-      <c r="D780" t="n">
-        <v>31</v>
-      </c>
-      <c r="E780" t="n">
+      <c r="C781" t="n">
+        <v>31</v>
+      </c>
+      <c r="D781" t="n">
+        <v>31</v>
+      </c>
+      <c r="E781" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor build script optimization
This resolves issue #32.
Correct null value handling in data processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E782"/>
+  <dimension ref="A1:E783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15283,20 +15283,39 @@
     </row>
     <row r="782">
       <c r="A782" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>31</v>
+      </c>
+      <c r="D782" t="n">
+        <v>31</v>
+      </c>
+      <c r="E782" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B782" t="inlineStr">
+      <c r="B783" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C782" t="n">
-        <v>31</v>
-      </c>
-      <c r="D782" t="n">
-        <v>31</v>
-      </c>
-      <c r="E782" t="n">
+      <c r="C783" t="n">
+        <v>31</v>
+      </c>
+      <c r="D783" t="n">
+        <v>31</v>
+      </c>
+      <c r="E783" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15311,7 +15330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E782"/>
+  <dimension ref="A1:E783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30163,20 +30182,39 @@
     </row>
     <row r="782">
       <c r="A782" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>31</v>
+      </c>
+      <c r="D782" t="n">
+        <v>31</v>
+      </c>
+      <c r="E782" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B782" t="inlineStr">
+      <c r="B783" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C782" t="n">
-        <v>31</v>
-      </c>
-      <c r="D782" t="n">
-        <v>31</v>
-      </c>
-      <c r="E782" t="n">
+      <c r="C783" t="n">
+        <v>31</v>
+      </c>
+      <c r="D783" t="n">
+        <v>31</v>
+      </c>
+      <c r="E783" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E784"/>
+  <dimension ref="A1:E785"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15321,20 +15321,39 @@
     </row>
     <row r="784">
       <c r="A784" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>31</v>
+      </c>
+      <c r="D784" t="n">
+        <v>31</v>
+      </c>
+      <c r="E784" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B784" t="inlineStr">
+      <c r="B785" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C784" t="n">
-        <v>31</v>
-      </c>
-      <c r="D784" t="n">
-        <v>31</v>
-      </c>
-      <c r="E784" t="n">
+      <c r="C785" t="n">
+        <v>31</v>
+      </c>
+      <c r="D785" t="n">
+        <v>31</v>
+      </c>
+      <c r="E785" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15349,7 +15368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E784"/>
+  <dimension ref="A1:E785"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30239,20 +30258,39 @@
     </row>
     <row r="784">
       <c r="A784" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>31</v>
+      </c>
+      <c r="D784" t="n">
+        <v>31</v>
+      </c>
+      <c r="E784" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B784" t="inlineStr">
+      <c r="B785" t="inlineStr">
         <is>
           <t>2026-08-21 07:35:18</t>
         </is>
       </c>
-      <c r="C784" t="n">
-        <v>31</v>
-      </c>
-      <c r="D784" t="n">
-        <v>31</v>
-      </c>
-      <c r="E784" t="n">
+      <c r="C785" t="n">
+        <v>31</v>
+      </c>
+      <c r="D785" t="n">
+        <v>31</v>
+      </c>
+      <c r="E785" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise login page ui elements
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E786"/>
+  <dimension ref="A1:E787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15359,20 +15359,39 @@
     </row>
     <row r="786">
       <c r="A786" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>31</v>
+      </c>
+      <c r="D786" t="n">
+        <v>31</v>
+      </c>
+      <c r="E786" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B786" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C786" t="n">
-        <v>31</v>
-      </c>
-      <c r="D786" t="n">
-        <v>31</v>
-      </c>
-      <c r="E786" t="n">
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>31</v>
+      </c>
+      <c r="D787" t="n">
+        <v>31</v>
+      </c>
+      <c r="E787" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15387,7 +15406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E786"/>
+  <dimension ref="A1:E787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30315,20 +30334,39 @@
     </row>
     <row r="786">
       <c r="A786" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>31</v>
+      </c>
+      <c r="D786" t="n">
+        <v>31</v>
+      </c>
+      <c r="E786" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B786" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C786" t="n">
-        <v>31</v>
-      </c>
-      <c r="D786" t="n">
-        <v>31</v>
-      </c>
-      <c r="E786" t="n">
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>31</v>
+      </c>
+      <c r="D787" t="n">
+        <v>31</v>
+      </c>
+      <c r="E787" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E788"/>
+  <dimension ref="A1:E789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15397,20 +15397,39 @@
     </row>
     <row r="788">
       <c r="A788" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>31</v>
+      </c>
+      <c r="D788" t="n">
+        <v>31</v>
+      </c>
+      <c r="E788" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B788" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C788" t="n">
-        <v>31</v>
-      </c>
-      <c r="D788" t="n">
-        <v>31</v>
-      </c>
-      <c r="E788" t="n">
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>31</v>
+      </c>
+      <c r="D789" t="n">
+        <v>31</v>
+      </c>
+      <c r="E789" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15425,7 +15444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E788"/>
+  <dimension ref="A1:E789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30391,20 +30410,39 @@
     </row>
     <row r="788">
       <c r="A788" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>31</v>
+      </c>
+      <c r="D788" t="n">
+        <v>31</v>
+      </c>
+      <c r="E788" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B788" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C788" t="n">
-        <v>31</v>
-      </c>
-      <c r="D788" t="n">
-        <v>31</v>
-      </c>
-      <c r="E788" t="n">
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>31</v>
+      </c>
+      <c r="D789" t="n">
+        <v>31</v>
+      </c>
+      <c r="E789" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add build script optimization
Fix race condition in concurrent processing.
Remove deprecated functions and clean up codebase.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E789"/>
+  <dimension ref="A1:E790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15416,20 +15416,39 @@
     </row>
     <row r="789">
       <c r="A789" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>31</v>
+      </c>
+      <c r="D789" t="n">
+        <v>31</v>
+      </c>
+      <c r="E789" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B789" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C789" t="n">
-        <v>31</v>
-      </c>
-      <c r="D789" t="n">
-        <v>31</v>
-      </c>
-      <c r="E789" t="n">
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>31</v>
+      </c>
+      <c r="D790" t="n">
+        <v>31</v>
+      </c>
+      <c r="E790" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15444,7 +15463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E789"/>
+  <dimension ref="A1:E790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30429,20 +30448,39 @@
     </row>
     <row r="789">
       <c r="A789" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>31</v>
+      </c>
+      <c r="D789" t="n">
+        <v>31</v>
+      </c>
+      <c r="E789" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B789" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C789" t="n">
-        <v>31</v>
-      </c>
-      <c r="D789" t="n">
-        <v>31</v>
-      </c>
-      <c r="E789" t="n">
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>31</v>
+      </c>
+      <c r="D790" t="n">
+        <v>31</v>
+      </c>
+      <c r="E790" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E790"/>
+  <dimension ref="A1:E791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15435,20 +15435,39 @@
     </row>
     <row r="790">
       <c r="A790" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>31</v>
+      </c>
+      <c r="D790" t="n">
+        <v>31</v>
+      </c>
+      <c r="E790" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B790" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C790" t="n">
-        <v>31</v>
-      </c>
-      <c r="D790" t="n">
-        <v>31</v>
-      </c>
-      <c r="E790" t="n">
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>31</v>
+      </c>
+      <c r="D791" t="n">
+        <v>31</v>
+      </c>
+      <c r="E791" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15463,7 +15482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E790"/>
+  <dimension ref="A1:E791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30467,20 +30486,39 @@
     </row>
     <row r="790">
       <c r="A790" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>31</v>
+      </c>
+      <c r="D790" t="n">
+        <v>31</v>
+      </c>
+      <c r="E790" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B790" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C790" t="n">
-        <v>31</v>
-      </c>
-      <c r="D790" t="n">
-        <v>31</v>
-      </c>
-      <c r="E790" t="n">
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>31</v>
+      </c>
+      <c r="D791" t="n">
+        <v>31</v>
+      </c>
+      <c r="E791" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize config file handling
This resolves issue #28.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E791"/>
+  <dimension ref="A1:E792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15454,20 +15454,39 @@
     </row>
     <row r="791">
       <c r="A791" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>31</v>
+      </c>
+      <c r="D791" t="n">
+        <v>31</v>
+      </c>
+      <c r="E791" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B791" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C791" t="n">
-        <v>31</v>
-      </c>
-      <c r="D791" t="n">
-        <v>31</v>
-      </c>
-      <c r="E791" t="n">
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>31</v>
+      </c>
+      <c r="D792" t="n">
+        <v>31</v>
+      </c>
+      <c r="E792" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15482,7 +15501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E791"/>
+  <dimension ref="A1:E792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30505,20 +30524,39 @@
     </row>
     <row r="791">
       <c r="A791" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>31</v>
+      </c>
+      <c r="D791" t="n">
+        <v>31</v>
+      </c>
+      <c r="E791" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B791" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C791" t="n">
-        <v>31</v>
-      </c>
-      <c r="D791" t="n">
-        <v>31</v>
-      </c>
-      <c r="E791" t="n">
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>31</v>
+      </c>
+      <c r="D792" t="n">
+        <v>31</v>
+      </c>
+      <c r="E792" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise user authentication module
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E792"/>
+  <dimension ref="A1:E793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15473,20 +15473,39 @@
     </row>
     <row r="792">
       <c r="A792" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>31</v>
+      </c>
+      <c r="D792" t="n">
+        <v>31</v>
+      </c>
+      <c r="E792" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B792" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C792" t="n">
-        <v>31</v>
-      </c>
-      <c r="D792" t="n">
-        <v>31</v>
-      </c>
-      <c r="E792" t="n">
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C793" t="n">
+        <v>31</v>
+      </c>
+      <c r="D793" t="n">
+        <v>31</v>
+      </c>
+      <c r="E793" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15501,7 +15520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E792"/>
+  <dimension ref="A1:E793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30543,20 +30562,39 @@
     </row>
     <row r="792">
       <c r="A792" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>31</v>
+      </c>
+      <c r="D792" t="n">
+        <v>31</v>
+      </c>
+      <c r="E792" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B792" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C792" t="n">
-        <v>31</v>
-      </c>
-      <c r="D792" t="n">
-        <v>31</v>
-      </c>
-      <c r="E792" t="n">
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C793" t="n">
+        <v>31</v>
+      </c>
+      <c r="D793" t="n">
+        <v>31</v>
+      </c>
+      <c r="E793" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance user authentication module
Correct null value handling in data processing.
Add missing documentation for the new API.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E794"/>
+  <dimension ref="A1:E795"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15511,20 +15511,39 @@
     </row>
     <row r="794">
       <c r="A794" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C794" t="n">
+        <v>31</v>
+      </c>
+      <c r="D794" t="n">
+        <v>31</v>
+      </c>
+      <c r="E794" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B794" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C794" t="n">
-        <v>31</v>
-      </c>
-      <c r="D794" t="n">
-        <v>31</v>
-      </c>
-      <c r="E794" t="n">
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>31</v>
+      </c>
+      <c r="D795" t="n">
+        <v>31</v>
+      </c>
+      <c r="E795" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15539,7 +15558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E794"/>
+  <dimension ref="A1:E795"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30619,20 +30638,39 @@
     </row>
     <row r="794">
       <c r="A794" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C794" t="n">
+        <v>31</v>
+      </c>
+      <c r="D794" t="n">
+        <v>31</v>
+      </c>
+      <c r="E794" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B794" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C794" t="n">
-        <v>31</v>
-      </c>
-      <c r="D794" t="n">
-        <v>31</v>
-      </c>
-      <c r="E794" t="n">
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>31</v>
+      </c>
+      <c r="D795" t="n">
+        <v>31</v>
+      </c>
+      <c r="E795" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove config file handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E795"/>
+  <dimension ref="A1:E796"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15530,20 +15530,39 @@
     </row>
     <row r="795">
       <c r="A795" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>31</v>
+      </c>
+      <c r="D795" t="n">
+        <v>31</v>
+      </c>
+      <c r="E795" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B795" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C795" t="n">
-        <v>31</v>
-      </c>
-      <c r="D795" t="n">
-        <v>31</v>
-      </c>
-      <c r="E795" t="n">
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>31</v>
+      </c>
+      <c r="D796" t="n">
+        <v>31</v>
+      </c>
+      <c r="E796" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15558,7 +15577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E795"/>
+  <dimension ref="A1:E796"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30657,20 +30676,39 @@
     </row>
     <row r="795">
       <c r="A795" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>31</v>
+      </c>
+      <c r="D795" t="n">
+        <v>31</v>
+      </c>
+      <c r="E795" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B795" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C795" t="n">
-        <v>31</v>
-      </c>
-      <c r="D795" t="n">
-        <v>31</v>
-      </c>
-      <c r="E795" t="n">
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>31</v>
+      </c>
+      <c r="D796" t="n">
+        <v>31</v>
+      </c>
+      <c r="E796" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E796"/>
+  <dimension ref="A1:E797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15549,20 +15549,39 @@
     </row>
     <row r="796">
       <c r="A796" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>31</v>
+      </c>
+      <c r="D796" t="n">
+        <v>31</v>
+      </c>
+      <c r="E796" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B796" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C796" t="n">
-        <v>31</v>
-      </c>
-      <c r="D796" t="n">
-        <v>31</v>
-      </c>
-      <c r="E796" t="n">
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>31</v>
+      </c>
+      <c r="D797" t="n">
+        <v>31</v>
+      </c>
+      <c r="E797" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15577,7 +15596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E796"/>
+  <dimension ref="A1:E797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30695,20 +30714,39 @@
     </row>
     <row r="796">
       <c r="A796" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>31</v>
+      </c>
+      <c r="D796" t="n">
+        <v>31</v>
+      </c>
+      <c r="E796" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B796" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C796" t="n">
-        <v>31</v>
-      </c>
-      <c r="D796" t="n">
-        <v>31</v>
-      </c>
-      <c r="E796" t="n">
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>31</v>
+      </c>
+      <c r="D797" t="n">
+        <v>31</v>
+      </c>
+      <c r="E797" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update api endpoint validation
Enhance test coverage to prevent regressions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E797"/>
+  <dimension ref="A1:E798"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15568,20 +15568,39 @@
     </row>
     <row r="797">
       <c r="A797" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>31</v>
+      </c>
+      <c r="D797" t="n">
+        <v>31</v>
+      </c>
+      <c r="E797" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B797" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C797" t="n">
-        <v>31</v>
-      </c>
-      <c r="D797" t="n">
-        <v>31</v>
-      </c>
-      <c r="E797" t="n">
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>31</v>
+      </c>
+      <c r="D798" t="n">
+        <v>31</v>
+      </c>
+      <c r="E798" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15596,7 +15615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E797"/>
+  <dimension ref="A1:E798"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30733,20 +30752,39 @@
     </row>
     <row r="797">
       <c r="A797" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>31</v>
+      </c>
+      <c r="D797" t="n">
+        <v>31</v>
+      </c>
+      <c r="E797" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B797" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C797" t="n">
-        <v>31</v>
-      </c>
-      <c r="D797" t="n">
-        <v>31</v>
-      </c>
-      <c r="E797" t="n">
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>31</v>
+      </c>
+      <c r="D798" t="n">
+        <v>31</v>
+      </c>
+      <c r="E798" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Upgrade build script optimization
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E798"/>
+  <dimension ref="A1:E799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15587,20 +15587,39 @@
     </row>
     <row r="798">
       <c r="A798" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>31</v>
+      </c>
+      <c r="D798" t="n">
+        <v>31</v>
+      </c>
+      <c r="E798" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B798" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C798" t="n">
-        <v>31</v>
-      </c>
-      <c r="D798" t="n">
-        <v>31</v>
-      </c>
-      <c r="E798" t="n">
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>31</v>
+      </c>
+      <c r="D799" t="n">
+        <v>31</v>
+      </c>
+      <c r="E799" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15615,7 +15634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E798"/>
+  <dimension ref="A1:E799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30771,20 +30790,39 @@
     </row>
     <row r="798">
       <c r="A798" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>31</v>
+      </c>
+      <c r="D798" t="n">
+        <v>31</v>
+      </c>
+      <c r="E798" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B798" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C798" t="n">
-        <v>31</v>
-      </c>
-      <c r="D798" t="n">
-        <v>31</v>
-      </c>
-      <c r="E798" t="n">
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>31</v>
+      </c>
+      <c r="D799" t="n">
+        <v>31</v>
+      </c>
+      <c r="E799" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E799"/>
+  <dimension ref="A1:E801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15606,20 +15606,58 @@
     </row>
     <row r="799">
       <c r="A799" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>31</v>
+      </c>
+      <c r="D799" t="n">
+        <v>31</v>
+      </c>
+      <c r="E799" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C800" t="n">
+        <v>31</v>
+      </c>
+      <c r="D800" t="n">
+        <v>31</v>
+      </c>
+      <c r="E800" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B799" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C799" t="n">
-        <v>31</v>
-      </c>
-      <c r="D799" t="n">
-        <v>31</v>
-      </c>
-      <c r="E799" t="n">
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C801" t="n">
+        <v>31</v>
+      </c>
+      <c r="D801" t="n">
+        <v>31</v>
+      </c>
+      <c r="E801" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15634,7 +15672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E799"/>
+  <dimension ref="A1:E801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30809,20 +30847,58 @@
     </row>
     <row r="799">
       <c r="A799" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>31</v>
+      </c>
+      <c r="D799" t="n">
+        <v>31</v>
+      </c>
+      <c r="E799" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C800" t="n">
+        <v>31</v>
+      </c>
+      <c r="D800" t="n">
+        <v>31</v>
+      </c>
+      <c r="E800" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B799" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C799" t="n">
-        <v>31</v>
-      </c>
-      <c r="D799" t="n">
-        <v>31</v>
-      </c>
-      <c r="E799" t="n">
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C801" t="n">
+        <v>31</v>
+      </c>
+      <c r="D801" t="n">
+        <v>31</v>
+      </c>
+      <c r="E801" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove file upload functionality
Simplify code structure to improve readability.
Improve performance by optimizing database queries.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E804"/>
+  <dimension ref="A1:E805"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15701,20 +15701,39 @@
     </row>
     <row r="804">
       <c r="A804" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C804" t="n">
+        <v>31</v>
+      </c>
+      <c r="D804" t="n">
+        <v>31</v>
+      </c>
+      <c r="E804" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B804" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C804" t="n">
-        <v>31</v>
-      </c>
-      <c r="D804" t="n">
-        <v>31</v>
-      </c>
-      <c r="E804" t="n">
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>31</v>
+      </c>
+      <c r="D805" t="n">
+        <v>31</v>
+      </c>
+      <c r="E805" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15729,7 +15748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E804"/>
+  <dimension ref="A1:E805"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30999,20 +31018,39 @@
     </row>
     <row r="804">
       <c r="A804" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C804" t="n">
+        <v>31</v>
+      </c>
+      <c r="D804" t="n">
+        <v>31</v>
+      </c>
+      <c r="E804" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B804" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C804" t="n">
-        <v>31</v>
-      </c>
-      <c r="D804" t="n">
-        <v>31</v>
-      </c>
-      <c r="E804" t="n">
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>31</v>
+      </c>
+      <c r="D805" t="n">
+        <v>31</v>
+      </c>
+      <c r="E805" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimize build script optimization
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E805"/>
+  <dimension ref="A1:E806"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15720,20 +15720,39 @@
     </row>
     <row r="805">
       <c r="A805" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>31</v>
+      </c>
+      <c r="D805" t="n">
+        <v>31</v>
+      </c>
+      <c r="E805" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B805" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C805" t="n">
-        <v>31</v>
-      </c>
-      <c r="D805" t="n">
-        <v>31</v>
-      </c>
-      <c r="E805" t="n">
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>31</v>
+      </c>
+      <c r="D806" t="n">
+        <v>31</v>
+      </c>
+      <c r="E806" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15748,7 +15767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E805"/>
+  <dimension ref="A1:E806"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31037,20 +31056,39 @@
     </row>
     <row r="805">
       <c r="A805" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>31</v>
+      </c>
+      <c r="D805" t="n">
+        <v>31</v>
+      </c>
+      <c r="E805" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B805" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C805" t="n">
-        <v>31</v>
-      </c>
-      <c r="D805" t="n">
-        <v>31</v>
-      </c>
-      <c r="E805" t="n">
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>31</v>
+      </c>
+      <c r="D806" t="n">
+        <v>31</v>
+      </c>
+      <c r="E806" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance unit test coverage
Add missing documentation for the new API.
This resolves issue #67.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E806"/>
+  <dimension ref="A1:E807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15739,20 +15739,39 @@
     </row>
     <row r="806">
       <c r="A806" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>31</v>
+      </c>
+      <c r="D806" t="n">
+        <v>31</v>
+      </c>
+      <c r="E806" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B806" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C806" t="n">
-        <v>31</v>
-      </c>
-      <c r="D806" t="n">
-        <v>31</v>
-      </c>
-      <c r="E806" t="n">
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C807" t="n">
+        <v>31</v>
+      </c>
+      <c r="D807" t="n">
+        <v>31</v>
+      </c>
+      <c r="E807" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15767,7 +15786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E806"/>
+  <dimension ref="A1:E807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31075,20 +31094,39 @@
     </row>
     <row r="806">
       <c r="A806" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>31</v>
+      </c>
+      <c r="D806" t="n">
+        <v>31</v>
+      </c>
+      <c r="E806" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B806" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C806" t="n">
-        <v>31</v>
-      </c>
-      <c r="D806" t="n">
-        <v>31</v>
-      </c>
-      <c r="E806" t="n">
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C807" t="n">
+        <v>31</v>
+      </c>
+      <c r="D807" t="n">
+        <v>31</v>
+      </c>
+      <c r="E807" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct csv module error handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E809"/>
+  <dimension ref="A1:E810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15796,20 +15796,39 @@
     </row>
     <row r="809">
       <c r="A809" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C809" t="n">
+        <v>31</v>
+      </c>
+      <c r="D809" t="n">
+        <v>31</v>
+      </c>
+      <c r="E809" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B809" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C809" t="n">
-        <v>31</v>
-      </c>
-      <c r="D809" t="n">
-        <v>31</v>
-      </c>
-      <c r="E809" t="n">
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>31</v>
+      </c>
+      <c r="D810" t="n">
+        <v>31</v>
+      </c>
+      <c r="E810" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15824,7 +15843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E809"/>
+  <dimension ref="A1:E810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31189,20 +31208,39 @@
     </row>
     <row r="809">
       <c r="A809" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C809" t="n">
+        <v>31</v>
+      </c>
+      <c r="D809" t="n">
+        <v>31</v>
+      </c>
+      <c r="E809" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B809" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C809" t="n">
-        <v>31</v>
-      </c>
-      <c r="D809" t="n">
-        <v>31</v>
-      </c>
-      <c r="E809" t="n">
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>31</v>
+      </c>
+      <c r="D810" t="n">
+        <v>31</v>
+      </c>
+      <c r="E810" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update database schema migration
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E810"/>
+  <dimension ref="A1:E811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15815,20 +15815,39 @@
     </row>
     <row r="810">
       <c r="A810" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>31</v>
+      </c>
+      <c r="D810" t="n">
+        <v>31</v>
+      </c>
+      <c r="E810" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B810" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C810" t="n">
-        <v>31</v>
-      </c>
-      <c r="D810" t="n">
-        <v>31</v>
-      </c>
-      <c r="E810" t="n">
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C811" t="n">
+        <v>31</v>
+      </c>
+      <c r="D811" t="n">
+        <v>31</v>
+      </c>
+      <c r="E811" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15843,7 +15862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E810"/>
+  <dimension ref="A1:E811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31227,20 +31246,39 @@
     </row>
     <row r="810">
       <c r="A810" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C810" t="n">
+        <v>31</v>
+      </c>
+      <c r="D810" t="n">
+        <v>31</v>
+      </c>
+      <c r="E810" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B810" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C810" t="n">
-        <v>31</v>
-      </c>
-      <c r="D810" t="n">
-        <v>31</v>
-      </c>
-      <c r="E810" t="n">
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C811" t="n">
+        <v>31</v>
+      </c>
+      <c r="D811" t="n">
+        <v>31</v>
+      </c>
+      <c r="E811" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct user authentication module
Update dependencies to their latest versions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E812"/>
+  <dimension ref="A1:E813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15853,20 +15853,39 @@
     </row>
     <row r="812">
       <c r="A812" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C812" t="n">
+        <v>31</v>
+      </c>
+      <c r="D812" t="n">
+        <v>31</v>
+      </c>
+      <c r="E812" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B812" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C812" t="n">
-        <v>31</v>
-      </c>
-      <c r="D812" t="n">
-        <v>31</v>
-      </c>
-      <c r="E812" t="n">
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C813" t="n">
+        <v>31</v>
+      </c>
+      <c r="D813" t="n">
+        <v>31</v>
+      </c>
+      <c r="E813" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15881,7 +15900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E812"/>
+  <dimension ref="A1:E813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31303,20 +31322,39 @@
     </row>
     <row r="812">
       <c r="A812" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C812" t="n">
+        <v>31</v>
+      </c>
+      <c r="D812" t="n">
+        <v>31</v>
+      </c>
+      <c r="E812" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B812" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C812" t="n">
-        <v>31</v>
-      </c>
-      <c r="D812" t="n">
-        <v>31</v>
-      </c>
-      <c r="E812" t="n">
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C813" t="n">
+        <v>31</v>
+      </c>
+      <c r="D813" t="n">
+        <v>31</v>
+      </c>
+      <c r="E813" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify unit test coverage
Apply code style fixes as per linter recommendations.
Enhance test coverage to prevent regressions.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E814"/>
+  <dimension ref="A1:E815"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15891,20 +15891,39 @@
     </row>
     <row r="814">
       <c r="A814" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C814" t="n">
+        <v>31</v>
+      </c>
+      <c r="D814" t="n">
+        <v>31</v>
+      </c>
+      <c r="E814" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B814" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C814" t="n">
-        <v>31</v>
-      </c>
-      <c r="D814" t="n">
-        <v>31</v>
-      </c>
-      <c r="E814" t="n">
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>31</v>
+      </c>
+      <c r="D815" t="n">
+        <v>31</v>
+      </c>
+      <c r="E815" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15919,7 +15938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E814"/>
+  <dimension ref="A1:E815"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31379,20 +31398,39 @@
     </row>
     <row r="814">
       <c r="A814" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C814" t="n">
+        <v>31</v>
+      </c>
+      <c r="D814" t="n">
+        <v>31</v>
+      </c>
+      <c r="E814" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B814" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C814" t="n">
-        <v>31</v>
-      </c>
-      <c r="D814" t="n">
-        <v>31</v>
-      </c>
-      <c r="E814" t="n">
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>31</v>
+      </c>
+      <c r="D815" t="n">
+        <v>31</v>
+      </c>
+      <c r="E815" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove security vulnerability checks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E815"/>
+  <dimension ref="A1:E816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15910,20 +15910,39 @@
     </row>
     <row r="815">
       <c r="A815" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>31</v>
+      </c>
+      <c r="D815" t="n">
+        <v>31</v>
+      </c>
+      <c r="E815" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B815" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C815" t="n">
-        <v>31</v>
-      </c>
-      <c r="D815" t="n">
-        <v>31</v>
-      </c>
-      <c r="E815" t="n">
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>31</v>
+      </c>
+      <c r="D816" t="n">
+        <v>31</v>
+      </c>
+      <c r="E816" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15938,7 +15957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E815"/>
+  <dimension ref="A1:E816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31417,20 +31436,39 @@
     </row>
     <row r="815">
       <c r="A815" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C815" t="n">
+        <v>31</v>
+      </c>
+      <c r="D815" t="n">
+        <v>31</v>
+      </c>
+      <c r="E815" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B815" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C815" t="n">
-        <v>31</v>
-      </c>
-      <c r="D815" t="n">
-        <v>31</v>
-      </c>
-      <c r="E815" t="n">
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>31</v>
+      </c>
+      <c r="D816" t="n">
+        <v>31</v>
+      </c>
+      <c r="E816" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor config file handling
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E816"/>
+  <dimension ref="A1:E817"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15929,20 +15929,39 @@
     </row>
     <row r="816">
       <c r="A816" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>31</v>
+      </c>
+      <c r="D816" t="n">
+        <v>31</v>
+      </c>
+      <c r="E816" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B816" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C816" t="n">
-        <v>31</v>
-      </c>
-      <c r="D816" t="n">
-        <v>31</v>
-      </c>
-      <c r="E816" t="n">
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C817" t="n">
+        <v>31</v>
+      </c>
+      <c r="D817" t="n">
+        <v>31</v>
+      </c>
+      <c r="E817" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15957,7 +15976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E816"/>
+  <dimension ref="A1:E817"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31455,20 +31474,39 @@
     </row>
     <row r="816">
       <c r="A816" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C816" t="n">
+        <v>31</v>
+      </c>
+      <c r="D816" t="n">
+        <v>31</v>
+      </c>
+      <c r="E816" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B816" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C816" t="n">
-        <v>31</v>
-      </c>
-      <c r="D816" t="n">
-        <v>31</v>
-      </c>
-      <c r="E816" t="n">
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C817" t="n">
+        <v>31</v>
+      </c>
+      <c r="D817" t="n">
+        <v>31</v>
+      </c>
+      <c r="E817" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E818"/>
+  <dimension ref="A1:E819"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15967,20 +15967,39 @@
     </row>
     <row r="818">
       <c r="A818" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C818" t="n">
+        <v>31</v>
+      </c>
+      <c r="D818" t="n">
+        <v>31</v>
+      </c>
+      <c r="E818" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B818" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C818" t="n">
-        <v>31</v>
-      </c>
-      <c r="D818" t="n">
-        <v>31</v>
-      </c>
-      <c r="E818" t="n">
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>31</v>
+      </c>
+      <c r="D819" t="n">
+        <v>31</v>
+      </c>
+      <c r="E819" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15995,7 +16014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E818"/>
+  <dimension ref="A1:E819"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31531,20 +31550,39 @@
     </row>
     <row r="818">
       <c r="A818" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C818" t="n">
+        <v>31</v>
+      </c>
+      <c r="D818" t="n">
+        <v>31</v>
+      </c>
+      <c r="E818" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B818" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C818" t="n">
-        <v>31</v>
-      </c>
-      <c r="D818" t="n">
-        <v>31</v>
-      </c>
-      <c r="E818" t="n">
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>31</v>
+      </c>
+      <c r="D819" t="n">
+        <v>31</v>
+      </c>
+      <c r="E819" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update csv module error handling
Address edge cases reported in user feedback.
Apply code style fixes as per linter recommendations.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E819"/>
+  <dimension ref="A1:E820"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15986,20 +15986,39 @@
     </row>
     <row r="819">
       <c r="A819" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>31</v>
+      </c>
+      <c r="D819" t="n">
+        <v>31</v>
+      </c>
+      <c r="E819" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B819" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C819" t="n">
-        <v>31</v>
-      </c>
-      <c r="D819" t="n">
-        <v>31</v>
-      </c>
-      <c r="E819" t="n">
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C820" t="n">
+        <v>31</v>
+      </c>
+      <c r="D820" t="n">
+        <v>31</v>
+      </c>
+      <c r="E820" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16014,7 +16033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E819"/>
+  <dimension ref="A1:E820"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31569,20 +31588,39 @@
     </row>
     <row r="819">
       <c r="A819" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C819" t="n">
+        <v>31</v>
+      </c>
+      <c r="D819" t="n">
+        <v>31</v>
+      </c>
+      <c r="E819" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B819" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C819" t="n">
-        <v>31</v>
-      </c>
-      <c r="D819" t="n">
-        <v>31</v>
-      </c>
-      <c r="E819" t="n">
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C820" t="n">
+        <v>31</v>
+      </c>
+      <c r="D820" t="n">
+        <v>31</v>
+      </c>
+      <c r="E820" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust image processing memory leaks
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E822"/>
+  <dimension ref="A1:E823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16043,20 +16043,39 @@
     </row>
     <row r="822">
       <c r="A822" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C822" t="n">
+        <v>31</v>
+      </c>
+      <c r="D822" t="n">
+        <v>31</v>
+      </c>
+      <c r="E822" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B822" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C822" t="n">
-        <v>31</v>
-      </c>
-      <c r="D822" t="n">
-        <v>31</v>
-      </c>
-      <c r="E822" t="n">
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>31</v>
+      </c>
+      <c r="D823" t="n">
+        <v>31</v>
+      </c>
+      <c r="E823" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16071,7 +16090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E822"/>
+  <dimension ref="A1:E823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31683,20 +31702,39 @@
     </row>
     <row r="822">
       <c r="A822" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C822" t="n">
+        <v>31</v>
+      </c>
+      <c r="D822" t="n">
+        <v>31</v>
+      </c>
+      <c r="E822" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B822" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C822" t="n">
-        <v>31</v>
-      </c>
-      <c r="D822" t="n">
-        <v>31</v>
-      </c>
-      <c r="E822" t="n">
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>31</v>
+      </c>
+      <c r="D823" t="n">
+        <v>31</v>
+      </c>
+      <c r="E823" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement navigation menu accessibility
Optimize image compression algorithm.
Fix various typos in comments and documentation.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E823"/>
+  <dimension ref="A1:E824"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16062,20 +16062,39 @@
     </row>
     <row r="823">
       <c r="A823" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>31</v>
+      </c>
+      <c r="D823" t="n">
+        <v>31</v>
+      </c>
+      <c r="E823" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B823" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C823" t="n">
-        <v>31</v>
-      </c>
-      <c r="D823" t="n">
-        <v>31</v>
-      </c>
-      <c r="E823" t="n">
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C824" t="n">
+        <v>31</v>
+      </c>
+      <c r="D824" t="n">
+        <v>31</v>
+      </c>
+      <c r="E824" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16090,7 +16109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E823"/>
+  <dimension ref="A1:E824"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31721,20 +31740,39 @@
     </row>
     <row r="823">
       <c r="A823" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C823" t="n">
+        <v>31</v>
+      </c>
+      <c r="D823" t="n">
+        <v>31</v>
+      </c>
+      <c r="E823" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B823" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C823" t="n">
-        <v>31</v>
-      </c>
-      <c r="D823" t="n">
-        <v>31</v>
-      </c>
-      <c r="E823" t="n">
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C824" t="n">
+        <v>31</v>
+      </c>
+      <c r="D824" t="n">
+        <v>31</v>
+      </c>
+      <c r="E824" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor logging system configuration
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E826"/>
+  <dimension ref="A1:E827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16119,20 +16119,39 @@
     </row>
     <row r="826">
       <c r="A826" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C826" t="n">
+        <v>31</v>
+      </c>
+      <c r="D826" t="n">
+        <v>31</v>
+      </c>
+      <c r="E826" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B826" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C826" t="n">
-        <v>31</v>
-      </c>
-      <c r="D826" t="n">
-        <v>31</v>
-      </c>
-      <c r="E826" t="n">
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>31</v>
+      </c>
+      <c r="D827" t="n">
+        <v>31</v>
+      </c>
+      <c r="E827" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16147,7 +16166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E826"/>
+  <dimension ref="A1:E827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31835,20 +31854,39 @@
     </row>
     <row r="826">
       <c r="A826" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C826" t="n">
+        <v>31</v>
+      </c>
+      <c r="D826" t="n">
+        <v>31</v>
+      </c>
+      <c r="E826" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B826" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C826" t="n">
-        <v>31</v>
-      </c>
-      <c r="D826" t="n">
-        <v>31</v>
-      </c>
-      <c r="E826" t="n">
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>31</v>
+      </c>
+      <c r="D827" t="n">
+        <v>31</v>
+      </c>
+      <c r="E827" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement unit test coverage
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E827"/>
+  <dimension ref="A1:E828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16138,20 +16138,39 @@
     </row>
     <row r="827">
       <c r="A827" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>31</v>
+      </c>
+      <c r="D827" t="n">
+        <v>31</v>
+      </c>
+      <c r="E827" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B827" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C827" t="n">
-        <v>31</v>
-      </c>
-      <c r="D827" t="n">
-        <v>31</v>
-      </c>
-      <c r="E827" t="n">
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C828" t="n">
+        <v>31</v>
+      </c>
+      <c r="D828" t="n">
+        <v>31</v>
+      </c>
+      <c r="E828" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16166,7 +16185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E827"/>
+  <dimension ref="A1:E828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31873,20 +31892,39 @@
     </row>
     <row r="827">
       <c r="A827" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C827" t="n">
+        <v>31</v>
+      </c>
+      <c r="D827" t="n">
+        <v>31</v>
+      </c>
+      <c r="E827" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B827" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C827" t="n">
-        <v>31</v>
-      </c>
-      <c r="D827" t="n">
-        <v>31</v>
-      </c>
-      <c r="E827" t="n">
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C828" t="n">
+        <v>31</v>
+      </c>
+      <c r="D828" t="n">
+        <v>31</v>
+      </c>
+      <c r="E828" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add data parsing logic
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E829"/>
+  <dimension ref="A1:E830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16176,20 +16176,39 @@
     </row>
     <row r="829">
       <c r="A829" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C829" t="n">
+        <v>31</v>
+      </c>
+      <c r="D829" t="n">
+        <v>31</v>
+      </c>
+      <c r="E829" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B829" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C829" t="n">
-        <v>31</v>
-      </c>
-      <c r="D829" t="n">
-        <v>31</v>
-      </c>
-      <c r="E829" t="n">
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>31</v>
+      </c>
+      <c r="D830" t="n">
+        <v>31</v>
+      </c>
+      <c r="E830" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16204,7 +16223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E829"/>
+  <dimension ref="A1:E830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31949,20 +31968,39 @@
     </row>
     <row r="829">
       <c r="A829" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C829" t="n">
+        <v>31</v>
+      </c>
+      <c r="D829" t="n">
+        <v>31</v>
+      </c>
+      <c r="E829" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B829" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C829" t="n">
-        <v>31</v>
-      </c>
-      <c r="D829" t="n">
-        <v>31</v>
-      </c>
-      <c r="E829" t="n">
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>31</v>
+      </c>
+      <c r="D830" t="n">
+        <v>31</v>
+      </c>
+      <c r="E830" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove logging system configuration
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E830"/>
+  <dimension ref="A1:E831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16195,20 +16195,39 @@
     </row>
     <row r="830">
       <c r="A830" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>31</v>
+      </c>
+      <c r="D830" t="n">
+        <v>31</v>
+      </c>
+      <c r="E830" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B830" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C830" t="n">
-        <v>31</v>
-      </c>
-      <c r="D830" t="n">
-        <v>31</v>
-      </c>
-      <c r="E830" t="n">
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C831" t="n">
+        <v>31</v>
+      </c>
+      <c r="D831" t="n">
+        <v>31</v>
+      </c>
+      <c r="E831" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16223,7 +16242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E830"/>
+  <dimension ref="A1:E831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31987,20 +32006,39 @@
     </row>
     <row r="830">
       <c r="A830" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C830" t="n">
+        <v>31</v>
+      </c>
+      <c r="D830" t="n">
+        <v>31</v>
+      </c>
+      <c r="E830" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B830" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C830" t="n">
-        <v>31</v>
-      </c>
-      <c r="D830" t="n">
-        <v>31</v>
-      </c>
-      <c r="E830" t="n">
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C831" t="n">
+        <v>31</v>
+      </c>
+      <c r="D831" t="n">
+        <v>31</v>
+      </c>
+      <c r="E831" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor user authentication module
Improve performance by optimizing database queries.
Fix race condition in concurrent processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E832"/>
+  <dimension ref="A1:E833"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16233,20 +16233,39 @@
     </row>
     <row r="832">
       <c r="A832" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C832" t="n">
+        <v>31</v>
+      </c>
+      <c r="D832" t="n">
+        <v>31</v>
+      </c>
+      <c r="E832" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B832" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C832" t="n">
-        <v>31</v>
-      </c>
-      <c r="D832" t="n">
-        <v>31</v>
-      </c>
-      <c r="E832" t="n">
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>31</v>
+      </c>
+      <c r="D833" t="n">
+        <v>31</v>
+      </c>
+      <c r="E833" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16261,7 +16280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E832"/>
+  <dimension ref="A1:E833"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32063,20 +32082,39 @@
     </row>
     <row r="832">
       <c r="A832" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C832" t="n">
+        <v>31</v>
+      </c>
+      <c r="D832" t="n">
+        <v>31</v>
+      </c>
+      <c r="E832" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B832" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C832" t="n">
-        <v>31</v>
-      </c>
-      <c r="D832" t="n">
-        <v>31</v>
-      </c>
-      <c r="E832" t="n">
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>31</v>
+      </c>
+      <c r="D833" t="n">
+        <v>31</v>
+      </c>
+      <c r="E833" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve error message display
Remove deprecated functions and clean up codebase.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E833"/>
+  <dimension ref="A1:E834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16252,20 +16252,39 @@
     </row>
     <row r="833">
       <c r="A833" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>31</v>
+      </c>
+      <c r="D833" t="n">
+        <v>31</v>
+      </c>
+      <c r="E833" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B833" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C833" t="n">
-        <v>31</v>
-      </c>
-      <c r="D833" t="n">
-        <v>31</v>
-      </c>
-      <c r="E833" t="n">
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C834" t="n">
+        <v>31</v>
+      </c>
+      <c r="D834" t="n">
+        <v>31</v>
+      </c>
+      <c r="E834" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16280,7 +16299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E833"/>
+  <dimension ref="A1:E834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32101,20 +32120,39 @@
     </row>
     <row r="833">
       <c r="A833" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C833" t="n">
+        <v>31</v>
+      </c>
+      <c r="D833" t="n">
+        <v>31</v>
+      </c>
+      <c r="E833" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B833" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C833" t="n">
-        <v>31</v>
-      </c>
-      <c r="D833" t="n">
-        <v>31</v>
-      </c>
-      <c r="E833" t="n">
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C834" t="n">
+        <v>31</v>
+      </c>
+      <c r="D834" t="n">
+        <v>31</v>
+      </c>
+      <c r="E834" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust unit test coverage
Add input validation for better security.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E838"/>
+  <dimension ref="A1:E839"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16347,20 +16347,39 @@
     </row>
     <row r="838">
       <c r="A838" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C838" t="n">
+        <v>31</v>
+      </c>
+      <c r="D838" t="n">
+        <v>31</v>
+      </c>
+      <c r="E838" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B838" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C838" t="n">
-        <v>31</v>
-      </c>
-      <c r="D838" t="n">
-        <v>31</v>
-      </c>
-      <c r="E838" t="n">
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C839" t="n">
+        <v>31</v>
+      </c>
+      <c r="D839" t="n">
+        <v>31</v>
+      </c>
+      <c r="E839" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16375,7 +16394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E838"/>
+  <dimension ref="A1:E839"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32291,20 +32310,39 @@
     </row>
     <row r="838">
       <c r="A838" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C838" t="n">
+        <v>31</v>
+      </c>
+      <c r="D838" t="n">
+        <v>31</v>
+      </c>
+      <c r="E838" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B838" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C838" t="n">
-        <v>31</v>
-      </c>
-      <c r="D838" t="n">
-        <v>31</v>
-      </c>
-      <c r="E838" t="n">
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C839" t="n">
+        <v>31</v>
+      </c>
+      <c r="D839" t="n">
+        <v>31</v>
+      </c>
+      <c r="E839" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add login page ui elements
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E841"/>
+  <dimension ref="A1:E842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16404,20 +16404,39 @@
     </row>
     <row r="841">
       <c r="A841" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C841" t="n">
+        <v>31</v>
+      </c>
+      <c r="D841" t="n">
+        <v>31</v>
+      </c>
+      <c r="E841" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B841" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C841" t="n">
-        <v>31</v>
-      </c>
-      <c r="D841" t="n">
-        <v>31</v>
-      </c>
-      <c r="E841" t="n">
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C842" t="n">
+        <v>31</v>
+      </c>
+      <c r="D842" t="n">
+        <v>31</v>
+      </c>
+      <c r="E842" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16432,7 +16451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E841"/>
+  <dimension ref="A1:E842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32405,20 +32424,39 @@
     </row>
     <row r="841">
       <c r="A841" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C841" t="n">
+        <v>31</v>
+      </c>
+      <c r="D841" t="n">
+        <v>31</v>
+      </c>
+      <c r="E841" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B841" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C841" t="n">
-        <v>31</v>
-      </c>
-      <c r="D841" t="n">
-        <v>31</v>
-      </c>
-      <c r="E841" t="n">
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C842" t="n">
+        <v>31</v>
+      </c>
+      <c r="D842" t="n">
+        <v>31</v>
+      </c>
+      <c r="E842" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix data parsing logic
Add missing documentation for the new API.
Simplify code structure to improve readability.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E851"/>
+  <dimension ref="A1:E852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16594,20 +16594,39 @@
     </row>
     <row r="851">
       <c r="A851" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C851" t="n">
+        <v>31</v>
+      </c>
+      <c r="D851" t="n">
+        <v>31</v>
+      </c>
+      <c r="E851" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B851" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C851" t="n">
-        <v>31</v>
-      </c>
-      <c r="D851" t="n">
-        <v>31</v>
-      </c>
-      <c r="E851" t="n">
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C852" t="n">
+        <v>31</v>
+      </c>
+      <c r="D852" t="n">
+        <v>31</v>
+      </c>
+      <c r="E852" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16622,7 +16641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E851"/>
+  <dimension ref="A1:E852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32785,20 +32804,39 @@
     </row>
     <row r="851">
       <c r="A851" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C851" t="n">
+        <v>31</v>
+      </c>
+      <c r="D851" t="n">
+        <v>31</v>
+      </c>
+      <c r="E851" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B851" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C851" t="n">
-        <v>31</v>
-      </c>
-      <c r="D851" t="n">
-        <v>31</v>
-      </c>
-      <c r="E851" t="n">
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C852" t="n">
+        <v>31</v>
+      </c>
+      <c r="D852" t="n">
+        <v>31</v>
+      </c>
+      <c r="E852" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance file upload functionality
Refactor legacy code to follow modern practices.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E855"/>
+  <dimension ref="A1:E856"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16670,20 +16670,39 @@
     </row>
     <row r="855">
       <c r="A855" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>31</v>
+      </c>
+      <c r="D855" t="n">
+        <v>31</v>
+      </c>
+      <c r="E855" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B855" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C855" t="n">
-        <v>31</v>
-      </c>
-      <c r="D855" t="n">
-        <v>31</v>
-      </c>
-      <c r="E855" t="n">
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>31</v>
+      </c>
+      <c r="D856" t="n">
+        <v>31</v>
+      </c>
+      <c r="E856" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16698,7 +16717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E855"/>
+  <dimension ref="A1:E856"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32937,20 +32956,39 @@
     </row>
     <row r="855">
       <c r="A855" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>31</v>
+      </c>
+      <c r="D855" t="n">
+        <v>31</v>
+      </c>
+      <c r="E855" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B855" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C855" t="n">
-        <v>31</v>
-      </c>
-      <c r="D855" t="n">
-        <v>31</v>
-      </c>
-      <c r="E855" t="n">
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>31</v>
+      </c>
+      <c r="D856" t="n">
+        <v>31</v>
+      </c>
+      <c r="E856" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add navigation menu accessibility
Add missing documentation for the new API.
Refactor legacy code to follow modern practices.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E856"/>
+  <dimension ref="A1:E857"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16689,20 +16689,39 @@
     </row>
     <row r="856">
       <c r="A856" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>31</v>
+      </c>
+      <c r="D856" t="n">
+        <v>31</v>
+      </c>
+      <c r="E856" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B856" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C856" t="n">
-        <v>31</v>
-      </c>
-      <c r="D856" t="n">
-        <v>31</v>
-      </c>
-      <c r="E856" t="n">
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>31</v>
+      </c>
+      <c r="D857" t="n">
+        <v>31</v>
+      </c>
+      <c r="E857" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16717,7 +16736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E856"/>
+  <dimension ref="A1:E857"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32975,20 +32994,39 @@
     </row>
     <row r="856">
       <c r="A856" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>31</v>
+      </c>
+      <c r="D856" t="n">
+        <v>31</v>
+      </c>
+      <c r="E856" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B856" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C856" t="n">
-        <v>31</v>
-      </c>
-      <c r="D856" t="n">
-        <v>31</v>
-      </c>
-      <c r="E856" t="n">
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>31</v>
+      </c>
+      <c r="D857" t="n">
+        <v>31</v>
+      </c>
+      <c r="E857" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove build script optimization
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E861"/>
+  <dimension ref="A1:E862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16784,20 +16784,39 @@
     </row>
     <row r="861">
       <c r="A861" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C861" t="n">
+        <v>31</v>
+      </c>
+      <c r="D861" t="n">
+        <v>31</v>
+      </c>
+      <c r="E861" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B861" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C861" t="n">
-        <v>31</v>
-      </c>
-      <c r="D861" t="n">
-        <v>31</v>
-      </c>
-      <c r="E861" t="n">
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>31</v>
+      </c>
+      <c r="D862" t="n">
+        <v>31</v>
+      </c>
+      <c r="E862" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16812,7 +16831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E861"/>
+  <dimension ref="A1:E862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33165,20 +33184,39 @@
     </row>
     <row r="861">
       <c r="A861" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C861" t="n">
+        <v>31</v>
+      </c>
+      <c r="D861" t="n">
+        <v>31</v>
+      </c>
+      <c r="E861" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B861" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C861" t="n">
-        <v>31</v>
-      </c>
-      <c r="D861" t="n">
-        <v>31</v>
-      </c>
-      <c r="E861" t="n">
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>31</v>
+      </c>
+      <c r="D862" t="n">
+        <v>31</v>
+      </c>
+      <c r="E862" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance api response formatting
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E862"/>
+  <dimension ref="A1:E863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16803,20 +16803,39 @@
     </row>
     <row r="862">
       <c r="A862" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>31</v>
+      </c>
+      <c r="D862" t="n">
+        <v>31</v>
+      </c>
+      <c r="E862" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B862" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C862" t="n">
-        <v>31</v>
-      </c>
-      <c r="D862" t="n">
-        <v>31</v>
-      </c>
-      <c r="E862" t="n">
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>31</v>
+      </c>
+      <c r="D863" t="n">
+        <v>31</v>
+      </c>
+      <c r="E863" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16831,7 +16850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E862"/>
+  <dimension ref="A1:E863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33203,20 +33222,39 @@
     </row>
     <row r="862">
       <c r="A862" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>31</v>
+      </c>
+      <c r="D862" t="n">
+        <v>31</v>
+      </c>
+      <c r="E862" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B862" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C862" t="n">
-        <v>31</v>
-      </c>
-      <c r="D862" t="n">
-        <v>31</v>
-      </c>
-      <c r="E862" t="n">
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>31</v>
+      </c>
+      <c r="D863" t="n">
+        <v>31</v>
+      </c>
+      <c r="E863" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve api response formatting
Fix race condition in concurrent processing.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E863"/>
+  <dimension ref="A1:E864"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16822,20 +16822,39 @@
     </row>
     <row r="863">
       <c r="A863" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>31</v>
+      </c>
+      <c r="D863" t="n">
+        <v>31</v>
+      </c>
+      <c r="E863" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B863" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C863" t="n">
-        <v>31</v>
-      </c>
-      <c r="D863" t="n">
-        <v>31</v>
-      </c>
-      <c r="E863" t="n">
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>31</v>
+      </c>
+      <c r="D864" t="n">
+        <v>31</v>
+      </c>
+      <c r="E864" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16850,7 +16869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E863"/>
+  <dimension ref="A1:E864"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33241,20 +33260,39 @@
     </row>
     <row r="863">
       <c r="A863" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>31</v>
+      </c>
+      <c r="D863" t="n">
+        <v>31</v>
+      </c>
+      <c r="E863" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B863" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C863" t="n">
-        <v>31</v>
-      </c>
-      <c r="D863" t="n">
-        <v>31</v>
-      </c>
-      <c r="E863" t="n">
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>31</v>
+      </c>
+      <c r="D864" t="n">
+        <v>31</v>
+      </c>
+      <c r="E864" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert unit test coverage
Add input validation for better security.
Refactor legacy code to follow modern practices.
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E864"/>
+  <dimension ref="A1:E865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16841,20 +16841,39 @@
     </row>
     <row r="864">
       <c r="A864" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>31</v>
+      </c>
+      <c r="D864" t="n">
+        <v>31</v>
+      </c>
+      <c r="E864" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B864" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C864" t="n">
-        <v>31</v>
-      </c>
-      <c r="D864" t="n">
-        <v>31</v>
-      </c>
-      <c r="E864" t="n">
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>31</v>
+      </c>
+      <c r="D865" t="n">
+        <v>31</v>
+      </c>
+      <c r="E865" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16869,7 +16888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E864"/>
+  <dimension ref="A1:E865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33279,20 +33298,39 @@
     </row>
     <row r="864">
       <c r="A864" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>31</v>
+      </c>
+      <c r="D864" t="n">
+        <v>31</v>
+      </c>
+      <c r="E864" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B864" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C864" t="n">
-        <v>31</v>
-      </c>
-      <c r="D864" t="n">
-        <v>31</v>
-      </c>
-      <c r="E864" t="n">
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>31</v>
+      </c>
+      <c r="D865" t="n">
+        <v>31</v>
+      </c>
+      <c r="E865" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise responsive design implementation
</commit_message>
<xml_diff>
--- a/Boddington_pwsTray_Database_update.xlsx
+++ b/Boddington_pwsTray_Database_update.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E866"/>
+  <dimension ref="A1:E867"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16879,20 +16879,39 @@
     </row>
     <row r="866">
       <c r="A866" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>31</v>
+      </c>
+      <c r="D866" t="n">
+        <v>31</v>
+      </c>
+      <c r="E866" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B866" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C866" t="n">
-        <v>31</v>
-      </c>
-      <c r="D866" t="n">
-        <v>31</v>
-      </c>
-      <c r="E866" t="n">
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>31</v>
+      </c>
+      <c r="D867" t="n">
+        <v>31</v>
+      </c>
+      <c r="E867" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16907,7 +16926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E866"/>
+  <dimension ref="A1:E867"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33355,20 +33374,39 @@
     </row>
     <row r="866">
       <c r="A866" s="2" t="n">
+        <v>46084.53551381944</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>31</v>
+      </c>
+      <c r="D866" t="n">
+        <v>31</v>
+      </c>
+      <c r="E866" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="n">
         <v>46084.53551382126</v>
       </c>
-      <c r="B866" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:18</t>
-        </is>
-      </c>
-      <c r="C866" t="n">
-        <v>31</v>
-      </c>
-      <c r="D866" t="n">
-        <v>31</v>
-      </c>
-      <c r="E866" t="n">
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>2026-08-21 07:35:18</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>31</v>
+      </c>
+      <c r="D867" t="n">
+        <v>31</v>
+      </c>
+      <c r="E867" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>